<commit_message>
Split consumables into cost types from the monthly stock-movement sheet (January model)
Add cogs_from_movement.py and the --movement option of the fill script: usage
net of internal returns mapped to Prostheses, Pharmacy, Laboratory, MS and OHF,
reconciled to the P&L cost of goods sold to the fils. January map regenerated;
January two-view model re-run and validated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types by month" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current implied" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumables detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current implied" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -758,7 +759,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>18064.5</v>
+        <v>17278.94</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>18659.88</v>
@@ -862,7 +863,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0</v>
+        <v>1252</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
@@ -914,7 +915,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>52796</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
@@ -966,7 +967,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>85932.98</v>
+        <v>31662.75</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>70788.92999999999</v>
@@ -1174,7 +1175,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>173786.41</v>
+        <v>174794.2</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>125812.55</v>
@@ -1610,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2069,7 +2070,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>14324.5</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>18259.88</v>
@@ -2105,7 +2106,7 @@
         <v>15194.75</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>195736.95</v>
+        <v>181412.45</v>
       </c>
     </row>
     <row r="8">
@@ -2201,7 +2202,7 @@
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>1870</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>200</v>
@@ -2237,178 +2238,178 @@
         <v>12557.75</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>54224.25</v>
+        <v>52354.25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -( Dr</t>
+          <t>Cost of Goods Sold (M01): Laboratory</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Laboratory</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — laboratory</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>clinical consumables issued to the dental surgeries</t>
+          <t>in-house lab materials (blocks, blanks, 3D inks, stone, milling tools) + external lab invoices</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>80969.67</v>
+        <v>15408.94</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>67171.58</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>70803.81</v>
+        <v>0</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>70803.81</v>
+        <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>63371.43</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>61129.96</v>
+        <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>46785.8</v>
+        <v>0</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>67034.7</v>
+        <v>0</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>62943.56</v>
+        <v>0</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>51591.7</v>
+        <v>0</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>39376.22</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>50594.58</v>
+        <v>0</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>732576.8199999999</v>
+        <v>15408.94</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
+          <t>Cost of Goods Sold (M01): Pharmacy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Direct — CSSD</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sterilisation and vital-signs consumables</t>
+          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4963.31</v>
+        <v>1252</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>3617.35</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>4137.43</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>4094.41</v>
+        <v>0</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>4096.91</v>
+        <v>0</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>4535.04</v>
+        <v>0</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>3033.61</v>
+        <v>0</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>3973.98</v>
+        <v>0</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>5793.45</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>9800.040000000001</v>
+        <v>0</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>57780.25</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Equipment Maintenanace</t>
+          <t>Cost of Goods Sold (M01): Prostheses</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — implants</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>maintenance of dental chairs and clinical equipment</t>
+          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1000</v>
+        <v>52796</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>2258.57</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>830</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>0</v>
@@ -2426,214 +2427,214 @@
         <v>0</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>1350</v>
+        <v>0</v>
       </c>
       <c r="P12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>5638.57</v>
+        <v>52796</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Depreciation: Machinery &amp; Equipment</t>
+          <t>Cost of Goods Sold: Consumables -( Dr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / imaging</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
+          <t>clinical consumables issued to the dental surgeries</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>10556.61</v>
+        <v>67171.58</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>10556.61</v>
+        <v>70803.81</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>10556.61</v>
+        <v>70803.81</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>10556.61</v>
+        <v>63371.43</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>10556.61</v>
+        <v>61129.96</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>10556.61</v>
+        <v>46785.8</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>10556.61</v>
+        <v>67034.7</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>10556.61</v>
+        <v>62943.56</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>10556.61</v>
+        <v>51591.7</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>10556.61</v>
+        <v>39376.22</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>10556.61</v>
+        <v>50594.58</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>126679.32</v>
+        <v>651607.15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education</t>
+          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Overhead — HR / IT</t>
+          <t>Direct — CSSD</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges</t>
+          <t>sterilisation and vital-signs consumables</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>28462.76</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>13180.32</v>
+        <v>3617.35</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>43627.94</v>
+        <v>4867.36</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>38711.94</v>
+        <v>4867.36</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>55516.92</v>
+        <v>4137.43</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>155175.22</v>
+        <v>4094.41</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>105124.99</v>
+        <v>4096.91</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>98355.2</v>
+        <v>4535.04</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>80992.27</v>
+        <v>3033.61</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>91500.75999999999</v>
+        <v>3973.98</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>46595.58</v>
+        <v>5793.45</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>132188.09</v>
+        <v>9800.040000000001</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>889431.99</v>
+        <v>52816.94</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Management</t>
+          <t>Cost of Goods Sold (M01): MS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Overhead — management</t>
+          <t>Direct — dental surgeries / CSSD</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>clinic management</t>
+          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>20000</v>
+        <v>31662.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>310000</v>
+        <v>31662.75</v>
       </c>
     </row>
     <row r="16">
@@ -2644,139 +2645,139 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses</t>
+          <t>Equipment Maintenanace</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees</t>
+          <t>maintenance of dental chairs and clinical equipment</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>44349.17</v>
+        <v>1000</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>12044.19</v>
+        <v>2258.57</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>12460.82</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>13383.95</v>
+        <v>830</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>20601.3</v>
+        <v>0</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>44034.76</v>
+        <v>0</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>13033.16</v>
+        <v>0</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>22175.9</v>
+        <v>0</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>18567.92</v>
+        <v>0</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>13508.57</v>
+        <v>1350</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>21037.68</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>18372.04</v>
+        <v>200</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>253569.46</v>
+        <v>5638.57</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>TB depreciation</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/RAP</t>
+          <t>Depreciation: Machinery &amp; Equipment</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Overhead — reception / patient administration</t>
+          <t>Direct — dental surgeries / imaging</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>reception and patient-administration staff</t>
+          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>11598</v>
+        <v>10556.61</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>12400</v>
+        <v>10556.61</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>12232</v>
+        <v>10556.61</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>10000</v>
+        <v>10556.61</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>14200</v>
+        <v>10556.61</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>13700</v>
+        <v>10556.61</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>13669</v>
+        <v>10556.61</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>14500</v>
+        <v>10556.61</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>15000</v>
+        <v>10556.61</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>21550</v>
+        <v>10556.61</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>21759</v>
+        <v>10556.61</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>22125</v>
+        <v>10556.61</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>182733</v>
+        <v>126679.32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: External</t>
+          <t>Staff Qualification And Education</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2786,52 +2787,52 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — HR / IT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>7600</v>
+        <v>28462.76</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>12690</v>
+        <v>13180.32</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>11520</v>
+        <v>43627.94</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>9505</v>
+        <v>38711.94</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>7800</v>
+        <v>55516.92</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>9070</v>
+        <v>155175.22</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>9700</v>
+        <v>105124.99</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>11596</v>
+        <v>98355.2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>16600</v>
+        <v>80992.27</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>15600</v>
+        <v>91500.75999999999</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>15600</v>
+        <v>46595.58</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>15600</v>
+        <v>132188.09</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>142881</v>
+        <v>889431.99</v>
       </c>
     </row>
     <row r="19">
@@ -2842,7 +2843,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /INS</t>
+          <t>Salaries &amp; Wages: Indirect /Management</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2852,52 +2853,52 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — management</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>insurance claims staff</t>
+          <t>clinic management</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>4400</v>
+        <v>20000</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>10567</v>
+        <v>20000</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>11500</v>
+        <v>28000</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>12000</v>
+        <v>27000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>10403</v>
+        <v>27000</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>11336</v>
+        <v>28000</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>10871</v>
+        <v>28000</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>11054</v>
+        <v>28000</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>11248</v>
+        <v>28000</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>11234</v>
+        <v>28000</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>11982.5</v>
+        <v>28000</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>121595.5</v>
+        <v>310000</v>
       </c>
     </row>
     <row r="20">
@@ -2908,7 +2909,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Clinic Rent</t>
+          <t>Legal &amp; Professional Expenses</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2918,63 +2919,63 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>7083.33</v>
+        <v>44349.17</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>7083.33</v>
+        <v>12044.19</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>7083.33</v>
+        <v>12460.82</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>7083.33</v>
+        <v>13383.95</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>7083.33</v>
+        <v>20601.3</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>7083.33</v>
+        <v>44034.76</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>7083.33</v>
+        <v>13033.16</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>7083.33</v>
+        <v>22175.9</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>7083.33</v>
+        <v>18567.92</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>7083.33</v>
+        <v>13508.57</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>7083.33</v>
+        <v>21037.68</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>7083.33</v>
+        <v>18372.04</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>84999.96000000001</v>
+        <v>253569.46</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dues &amp; Subscriptions</t>
+          <t>Salaries &amp; Wages: Indirect/RAP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2984,63 +2985,63 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Overhead — IT / administration</t>
+          <t>Overhead — reception / patient administration</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>software subscriptions, memberships</t>
+          <t>reception and patient-administration staff</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>5585</v>
+        <v>11598</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>9203.280000000001</v>
+        <v>12400</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>8414.280000000001</v>
+        <v>12232</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>6503.7</v>
+        <v>14200</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>10028.04</v>
+        <v>13700</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>99.54000000000001</v>
+        <v>13669</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>1842.43</v>
+        <v>14500</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>15774.05</v>
+        <v>15000</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>6523.81</v>
+        <v>21550</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>8884.18</v>
+        <v>21759</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>5667.86</v>
+        <v>22125</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>80526.17</v>
+        <v>182733</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Finance Charges</t>
+          <t>Salaries &amp; Wages: External</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3055,47 +3056,47 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>bank and card charges</t>
+          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>6820.88</v>
+        <v>7600</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>6684.05</v>
+        <v>12690</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>9269.73</v>
+        <v>11520</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>5865.9</v>
+        <v>9505</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>5876.86</v>
+        <v>7800</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>4410.88</v>
+        <v>9070</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>3220.43</v>
+        <v>9700</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>4136.27</v>
+        <v>11596</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>4080.58</v>
+        <v>16600</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>4032.3</v>
+        <v>15600</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>4905.68</v>
+        <v>15600</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>3702.29</v>
+        <v>15600</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>63005.85</v>
+        <v>142881</v>
       </c>
     </row>
     <row r="23">
@@ -3106,7 +3107,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Purchase</t>
+          <t>Salaries &amp; Wages: Indirect /INS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3116,52 +3117,52 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>purchasing</t>
+          <t>insurance claims staff</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>5000</v>
+        <v>4400</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>5000</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>5000</v>
+        <v>10567</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>5000</v>
+        <v>11500</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>4458</v>
+        <v>12000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>5000</v>
+        <v>10403</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>5000</v>
+        <v>11336</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>5000</v>
+        <v>10871</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>5000</v>
+        <v>11054</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>5000</v>
+        <v>11248</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>4758</v>
+        <v>11234</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>4958.33</v>
+        <v>11982.5</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>59174.33</v>
+        <v>121595.5</v>
       </c>
     </row>
     <row r="24">
@@ -3172,7 +3173,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Utilities Expenses</t>
+          <t>Clinic Rent</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3187,47 +3188,47 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ADDC electricity/water, Etisalat telephone and internet</t>
+          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>4780.25</v>
+        <v>7083.33</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>4568.37</v>
+        <v>7083.33</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>4510.14</v>
+        <v>7083.33</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>4191.56</v>
+        <v>7083.33</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>8334.92</v>
+        <v>7083.33</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>4350.26</v>
+        <v>7083.33</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>4242.75</v>
+        <v>7083.33</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>4051.47</v>
+        <v>7083.33</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>4127.37</v>
+        <v>7083.33</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>4358.95</v>
+        <v>7083.33</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>4242.9</v>
+        <v>7083.33</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>4322.62</v>
+        <v>7083.33</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>56081.56</v>
+        <v>84999.96000000001</v>
       </c>
     </row>
     <row r="25">
@@ -3238,7 +3239,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3248,63 +3249,63 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — IT / administration</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Meta/WhatsApp API, Adobe, promotions</t>
+          <t>software subscriptions, memberships</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>5820.11</v>
+        <v>5585</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>2380.86</v>
+        <v>9203.280000000001</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>4382.51</v>
+        <v>8414.280000000001</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>4044.86</v>
+        <v>2000</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>4998.58</v>
+        <v>6503.7</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>8392.940000000001</v>
+        <v>10028.04</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>3713.11</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>5896.89</v>
+        <v>1842.43</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>2707.23</v>
+        <v>15774.05</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>1973.75</v>
+        <v>6523.81</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>8600.299999999999</v>
+        <v>8884.18</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>2478.75</v>
+        <v>5667.86</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>55389.89</v>
+        <v>80526.17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/Accounts</t>
+          <t>Finance Charges</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3319,58 +3320,58 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>accounts</t>
+          <t>bank and card charges</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>4645</v>
+        <v>6820.88</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>3355</v>
+        <v>6684.05</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>4500</v>
+        <v>9269.73</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>4000</v>
+        <v>5865.9</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>3956</v>
+        <v>5876.86</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>4391</v>
+        <v>4410.88</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>4938</v>
+        <v>3220.43</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>3975</v>
+        <v>4136.27</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>4090</v>
+        <v>4080.58</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>4016</v>
+        <v>4032.3</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>4658</v>
+        <v>4905.68</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>4656.25</v>
+        <v>3702.29</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>51180.25</v>
+        <v>63005.85</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Salaries &amp; Wages: Indirect /Purchase</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3385,47 +3386,47 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman)</t>
+          <t>purchasing</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5939.4</v>
+        <v>5000</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>5974.65</v>
+        <v>5000</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>5974.65</v>
+        <v>5000</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>5974.65</v>
+        <v>5000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>5995.8</v>
+        <v>4458</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>5995.8</v>
+        <v>5000</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>4564.01</v>
+        <v>5000</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>1833.1</v>
+        <v>5000</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>1974.43</v>
+        <v>5000</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>1974.43</v>
+        <v>5000</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>2038.43</v>
+        <v>4758</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>2169.92</v>
+        <v>4958.33</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>50409.27</v>
+        <v>59174.33</v>
       </c>
     </row>
     <row r="28">
@@ -3436,7 +3437,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Repair &amp; Maintenance Expenses</t>
+          <t>Utilities Expenses</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3451,47 +3452,47 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>general premises maintenance supplies and works</t>
+          <t>ADDC electricity/water, Etisalat telephone and internet</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>3948.75</v>
+        <v>4780.25</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>701.2</v>
+        <v>4568.37</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1519</v>
+        <v>4510.14</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>2904.65</v>
+        <v>4191.56</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>418.3</v>
+        <v>8334.92</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>3500</v>
+        <v>4350.26</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>579.13</v>
+        <v>4242.75</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>3615.85</v>
+        <v>4051.47</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>4075.55</v>
+        <v>4127.37</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>4223.2</v>
+        <v>4358.95</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>2824</v>
+        <v>4242.9</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>704.67</v>
+        <v>4322.62</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>29014.3</v>
+        <v>56081.56</v>
       </c>
     </row>
     <row r="29">
@@ -3502,7 +3503,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Travelling &amp; Transportation</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3517,58 +3518,58 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>taxis, parking, petrol, car wash</t>
+          <t>Meta/WhatsApp API, Adobe, promotions</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1620.78</v>
+        <v>5820.11</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>2671.44</v>
+        <v>2380.86</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1406.51</v>
+        <v>4382.51</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>2252.91</v>
+        <v>4044.86</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>2285.53</v>
+        <v>4998.58</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1225.52</v>
+        <v>8392.940000000001</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>5340.97</v>
+        <v>3713.11</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>1464.2</v>
+        <v>5896.89</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>1523</v>
+        <v>2707.23</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>3348</v>
+        <v>1973.75</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>2184.07</v>
+        <v>8600.299999999999</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>2346.5</v>
+        <v>2478.75</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>27669.43</v>
+        <v>55389.89</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fines</t>
+          <t>Salaries &amp; Wages: Indirect/Accounts</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3583,47 +3584,47 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+          <t>accounts</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>1635</v>
+        <v>4645</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>263</v>
+        <v>3355</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>1278</v>
+        <v>4000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0</v>
+        <v>3956</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1031</v>
+        <v>4391</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0</v>
+        <v>4938</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>8435.120000000001</v>
+        <v>3975</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>1503</v>
+        <v>4090</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0</v>
+        <v>4016</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>2242.91</v>
+        <v>4658</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>625</v>
+        <v>4656.25</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>17013.03</v>
+        <v>51180.25</v>
       </c>
     </row>
     <row r="31">
@@ -3634,7 +3635,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pantry</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3644,52 +3645,52 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+          <t>prepaid insurance amortised (staff medical insurance, Daman)</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1576.08</v>
+        <v>5939.4</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>1074.12</v>
+        <v>5974.65</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>748.9299999999999</v>
+        <v>5974.65</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>1483.1</v>
+        <v>5974.65</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>705.55</v>
+        <v>5995.8</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1314.1</v>
+        <v>5995.8</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>1310.92</v>
+        <v>4564.01</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>1821.61</v>
+        <v>1833.1</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>1056.15</v>
+        <v>1974.43</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>1638.4</v>
+        <v>1974.43</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>1660.35</v>
+        <v>2038.43</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>752.78</v>
+        <v>2169.92</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>15142.09</v>
+        <v>50409.27</v>
       </c>
     </row>
     <row r="32">
@@ -3700,7 +3701,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Repair &amp; Maintenance Expenses</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3710,52 +3711,52 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>courier, flags/badges, miscellaneous</t>
+          <t>general premises maintenance supplies and works</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>2138.76</v>
+        <v>3948.75</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1089.69</v>
+        <v>701.2</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1123.01</v>
+        <v>1519</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>3789.07</v>
+        <v>2904.65</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>1320.49</v>
+        <v>418.3</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>989.6799999999999</v>
+        <v>3500</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>1127.98</v>
+        <v>579.13</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>1253.75</v>
+        <v>3615.85</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>508.94</v>
+        <v>4075.55</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>264.83</v>
+        <v>4223.2</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>316.45</v>
+        <v>2824</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>88.53</v>
+        <v>704.67</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>14011.18</v>
+        <v>29014.3</v>
       </c>
     </row>
     <row r="33">
@@ -3766,7 +3767,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Travelling &amp; Transportation</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3781,47 +3782,47 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>stationery, printer ink, newspapers</t>
+          <t>taxis, parking, petrol, car wash</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>783.13</v>
+        <v>1620.78</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>449.05</v>
+        <v>2671.44</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>373</v>
+        <v>1406.51</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>1618.98</v>
+        <v>2252.91</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>404.77</v>
+        <v>2285.53</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1228.67</v>
+        <v>1225.52</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>340.61</v>
+        <v>5340.97</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>481.01</v>
+        <v>1464.2</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>1156.65</v>
+        <v>1523</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>440.57</v>
+        <v>3348</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>237.4</v>
+        <v>2184.07</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>375.55</v>
+        <v>2346.5</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>7889.39</v>
+        <v>27669.43</v>
       </c>
     </row>
     <row r="34">
@@ -3832,7 +3833,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Claim Rejection</t>
+          <t>Fines</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3842,63 +3843,63 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>written-off rejected claims</t>
+          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>0</v>
+        <v>1635</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0</v>
+        <v>263</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>844.2</v>
+        <v>0</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0</v>
+        <v>1278</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>245</v>
+        <v>1031</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0</v>
+        <v>8435.120000000001</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>1005</v>
+        <v>1503</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>-32</v>
+        <v>0</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>1235</v>
+        <v>2242.91</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>105</v>
+        <v>625</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>3402.2</v>
+        <v>17013.03</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect it</t>
+          <t>Pantry</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3908,63 +3909,63 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Overhead — IT</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0</v>
+        <v>1576.08</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0</v>
+        <v>1074.12</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0</v>
+        <v>748.9299999999999</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>0</v>
+        <v>1483.1</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0</v>
+        <v>705.55</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0</v>
+        <v>1314.1</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>0</v>
+        <v>1310.92</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0</v>
+        <v>1821.61</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0</v>
+        <v>1056.15</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0</v>
+        <v>1638.4</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>0</v>
+        <v>1660.35</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>0</v>
+        <v>752.78</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>0</v>
+        <v>15142.09</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+          <t>Other Expenses</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3974,118 +3975,118 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Overhead — HR</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>courier, flags/badges, miscellaneous</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>0</v>
+        <v>2138.76</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>0</v>
+        <v>1089.69</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0</v>
+        <v>1123.01</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0</v>
+        <v>3789.07</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0</v>
+        <v>1320.49</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0</v>
+        <v>989.6799999999999</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0</v>
+        <v>1127.98</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0</v>
+        <v>1253.75</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0</v>
+        <v>508.94</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0</v>
+        <v>264.83</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>0</v>
+        <v>316.45</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>0</v>
+        <v>88.53</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>0</v>
+        <v>14011.18</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Depreciation: furniture, office equipment, computers, software</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OHDepreciation</t>
+          <t>OHF</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Overhead — facility / IT</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+          <t>stationery, printer ink, newspapers</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>2524.8</v>
+        <v>783.13</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>2524.8</v>
+        <v>449.05</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>2524.8</v>
+        <v>373</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>2524.8</v>
+        <v>1618.98</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>2524.8</v>
+        <v>404.77</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>2524.8</v>
+        <v>1228.67</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>2524.8</v>
+        <v>340.61</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>2524.8</v>
+        <v>481.01</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>2524.8</v>
+        <v>1156.65</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>2524.8</v>
+        <v>440.57</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>2524.8</v>
+        <v>237.4</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>2524.8</v>
+        <v>375.55</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>30297.6</v>
+        <v>7889.39</v>
       </c>
     </row>
     <row r="38">
@@ -4096,176 +4097,506 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>Claim Rejection</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Overhead — patient administration</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>written-off rejected claims</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>844.2</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>245</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>1005</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>-32</v>
+      </c>
+      <c r="P38" s="3" t="n">
+        <v>1235</v>
+      </c>
+      <c r="Q38" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="R38" s="3" t="n">
+        <v>3402.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Stock movement</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Cost of Goods Sold (M01): OHF</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Overhead — back office</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>pantry and stationery issued from stock</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>1007.8</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="3" t="n">
+        <v>1007.8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Salary sheet</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Salaries &amp; Wages: Indirect it</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Overhead — IT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Salary sheet</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Overhead — HR</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TB depreciation</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Depreciation: furniture, office equipment, computers, software</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Overhead — facility / IT</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="M42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="P42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="Q42" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>30297.6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Third Party &amp; Professional Services</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>OHC</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Overhead — shared services</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>MySmyle Company EMR subscription, management consultancy and IT services (25,000/month) + Calibrate/Platform Technologies: services charged by a sister company = corporate/shared-services overhead</t>
         </is>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F43" s="3" t="n">
         <v>8317</v>
       </c>
-      <c r="G38" s="3" t="n">
+      <c r="G43" s="3" t="n">
         <v>37300</v>
       </c>
-      <c r="H38" s="3" t="n">
+      <c r="H43" s="3" t="n">
         <v>62270</v>
       </c>
-      <c r="I38" s="3" t="n">
+      <c r="I43" s="3" t="n">
         <v>66480.95</v>
       </c>
-      <c r="J38" s="3" t="n">
+      <c r="J43" s="3" t="n">
         <v>2500</v>
       </c>
-      <c r="K38" s="3" t="n">
+      <c r="K43" s="3" t="n">
         <v>37375.73</v>
       </c>
-      <c r="L38" s="3" t="n">
+      <c r="L43" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="M38" s="3" t="n">
+      <c r="M43" s="3" t="n">
         <v>27500</v>
       </c>
-      <c r="N38" s="3" t="n">
+      <c r="N43" s="3" t="n">
         <v>28000</v>
       </c>
-      <c r="O38" s="3" t="n">
+      <c r="O43" s="3" t="n">
         <v>25500</v>
       </c>
-      <c r="P38" s="3" t="n">
+      <c r="P43" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="Q38" s="3" t="n">
+      <c r="Q43" s="3" t="n">
         <v>25104.5</v>
       </c>
-      <c r="R38" s="3" t="n">
+      <c r="R43" s="3" t="n">
         <v>370348.18</v>
       </c>
     </row>
-    <row r="39">
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
-      <c r="Q39" s="3" t="n"/>
-      <c r="R39" s="3" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="4" t="inlineStr">
+    <row r="44">
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="n"/>
+      <c r="N44" s="3" t="n"/>
+      <c r="O44" s="3" t="n"/>
+      <c r="P44" s="3" t="n"/>
+      <c r="Q44" s="3" t="n"/>
+      <c r="R44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>TOTAL mapped</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="5" t="n">
-        <v>511302.29</v>
-      </c>
-      <c r="G40" s="5" t="n">
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="5" t="n">
+        <v>511302.3</v>
+      </c>
+      <c r="G45" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H40" s="5" t="n">
+      <c r="H45" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I40" s="5" t="n">
+      <c r="I45" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J40" s="5" t="n">
+      <c r="J45" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K40" s="5" t="n">
+      <c r="K45" s="5" t="n">
         <v>616494.08</v>
       </c>
-      <c r="L40" s="5" t="n">
+      <c r="L45" s="5" t="n">
         <v>480166.81</v>
       </c>
-      <c r="M40" s="5" t="n">
+      <c r="M45" s="5" t="n">
         <v>526990.09</v>
       </c>
-      <c r="N40" s="5" t="n">
+      <c r="N45" s="5" t="n">
         <v>509542.04</v>
       </c>
-      <c r="O40" s="5" t="n">
+      <c r="O45" s="5" t="n">
         <v>546725.96</v>
       </c>
-      <c r="P40" s="5" t="n">
+      <c r="P45" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q40" s="5" t="n">
+      <c r="Q45" s="5" t="n">
         <v>623033.72</v>
       </c>
-      <c r="R40" s="5" t="n">
-        <v>6453401.9</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="R45" s="5" t="n">
+        <v>6453401.91</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Ledger (locked)</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="5" t="n">
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="5" t="n">
         <v>511302.3</v>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G46" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H46" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I46" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J46" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K41" s="5" t="n">
+      <c r="K46" s="5" t="n">
         <v>616494.09</v>
       </c>
-      <c r="L41" s="5" t="n">
+      <c r="L46" s="5" t="n">
         <v>480166.82</v>
       </c>
-      <c r="M41" s="5" t="n">
+      <c r="M46" s="5" t="n">
         <v>526990.1</v>
       </c>
-      <c r="N41" s="5" t="n">
+      <c r="N46" s="5" t="n">
         <v>509542.05</v>
       </c>
-      <c r="O41" s="5" t="n">
+      <c r="O46" s="5" t="n">
         <v>546725.98</v>
       </c>
-      <c r="P41" s="5" t="n">
+      <c r="P46" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q41" s="5" t="n">
+      <c r="Q46" s="5" t="n">
         <v>623033.73</v>
       </c>
-      <c r="R41" s="5" t="n">
+      <c r="R46" s="5" t="n">
         <v>6453401.98</v>
       </c>
     </row>
@@ -4280,7 +4611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -4331,7 +4662,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Overhead ratio by month: 01 36.1%, 02 31.1%, 03 38.0%, 04 44.7%, 05 39.8%, 06 58.1%, 07 52.1%, 08 50.6%, 09 50.3%, 10 46.5%, 11 46.1%, 12 47.5%; FY2025 45.2% (DOH band 20% to under 50%)</t>
+          <t>Overhead ratio by month: 01 36.3%, 02 31.1%, 03 38.0%, 04 44.7%, 05 39.8%, 06 58.1%, 07 52.1%, 08 50.6%, 09 50.3%, 10 46.5%, 11 46.1%, 12 47.5%; FY2025 45.2% (DOH band 20% to under 50%)</t>
         </is>
       </c>
     </row>
@@ -4345,131 +4676,110 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 1: split 102127.48 != Monthly 102127.49</t>
+          <t>Cost of Goods Sold month 2: split 89248.81 != Monthly 89248.80</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 2: split 89248.81 != Monthly 89248.80</t>
+          <t>Cost of Goods Sold month 3: split 104387.41 != Monthly 104387.40</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 3: split 104387.41 != Monthly 104387.40</t>
+          <t>Cost of Goods Sold month 4: split 98837.41 != Monthly 98837.40</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 4: split 98837.41 != Monthly 98837.40</t>
+          <t>Cost of Goods Sold month 5: split 82250.54 != Monthly 82250.53</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 5: split 82250.54 != Monthly 82250.53</t>
+          <t>month 6: mapped total 616494.08 != ledger 616494.09 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>month 1: mapped total 511302.29 != ledger 511302.30 (-0.01)</t>
+          <t>month 7: mapped total 480166.81 != ledger 480166.82 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>month 6: mapped total 616494.08 != ledger 616494.09 (-0.01)</t>
+          <t>month 8: mapped total 526990.09 != ledger 526990.10 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>month 7: mapped total 480166.81 != ledger 480166.82 (-0.01)</t>
+          <t>month 9: mapped total 509542.04 != ledger 509542.05 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>month 8: mapped total 526990.09 != ledger 526990.10 (-0.01)</t>
+          <t>month 10: mapped total 546725.96 != ledger 546725.98 (-0.02)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>month 9: mapped total 509542.04 != ledger 509542.05 (-0.01)</t>
+          <t>month 12: mapped total 623033.72 != ledger 623033.73 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>month 10: mapped total 546725.96 != ledger 546725.98 (-0.02)</t>
+          <t>month 6: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>month 12: mapped total 623033.72 != ledger 623033.73 (-0.01)</t>
+          <t>month 7: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>month 1: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 8: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>month 6: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 9: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>month 7: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 10: +0.02 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
-        <is>
-          <t>month 8: +0.01 added to OHF to tie to the locked ledger</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>month 9: +0.01 added to OHF to tie to the locked ledger</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>month 10: +0.02 added to OHF to tie to the locked ledger</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
         <is>
           <t>month 12: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
@@ -4481,6 +4791,268 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="150" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Stock movement -&gt; cost type (usage net of internal returns; exchanges cancel; external lab from the P&amp;L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           130.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,889.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           03- Dental Blanks                                   1,875.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              5,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   58.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        985.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessories     1,601.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   05- Medical Electronic Devices (Restorative, Perio, Endo, Implants, Ortho…)    5,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo, Implants,Ortho…)       83.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   345.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,993.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,477.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,007.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        540.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   338.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          806.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,552.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            756.62</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      4,441.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,630.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     710.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   690.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,700.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            90.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   847.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  160.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                682.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         570.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               27,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           3,699.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       6,652.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               960.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             13,985.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Movement Jan 2025: Laboratory  External LAB (P&amp;L line, not stock)                                            1,870.00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4590,7 +5162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Ledger-driven two-view engine: buckets derived from cost types by the 10 Oct 2026 rulings
Replace the bucket-anchored fit with a claim x cost-type fit seeded by the
allocation table's own cells; buckets follow fixed shares (Anaesthesia = drugs
+ 2% dentists + 1% nurses; Imaging = 4% nurses + 4% equipment depreciation +
imaging supplies; Laboratory = lab cost + lab technicians; Prosthesis =
implants; Dental the rest with overheads). Bucket-share sheet written from the
payroll split; January model re-run, validated and reported.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumables detail" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current implied" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket shares" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -77,6 +78,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6108,4 +6110,334 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>M06</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>M07</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>M08</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>M09</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWAllied lab share</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>0.5053003533568905</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0.4448850118953211</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0.4457201678676063</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0.3190151911995809</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0.4188792837936224</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>0.3457943925233645</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0.5269311346894641</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>0.4827586206896552</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>0.3922371668851912</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>0.5061071497246054</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>0.6062556139336295</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>laboratory technicians / (laboratory technicians + CSSD technicians), Salary sheet; drives the Laboratory bucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc to Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ruling 10 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWNurs to Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ruling 10 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SWNurs to Imaging</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>ruling 10 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Depreciation to Imaging</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ruling 10 Oct 2026 (equipment depreciation; OPG / X-ray units)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ruling: no laboratory — every prosthesis code is Prostheses; reroute lab cost, pre-assign prostheses and dental technicians on prosthesis claims; adopt the Finance Director's account-level splits
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Salaries and wages — allied health incl. technicians (hygienists, radiographers, lab technicians)</t>
+          <t>Salaries and wages — allied health incl. technicians (CSSD technicians; dental technicians, routed to the Prosthesis bucket)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -757,44 +757,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Laboratory supplies and outsourced laboratory invoices (dental lab work)</t>
+          <t>Pathology laboratory supplies — none: the clinic has no laboratory (ruling 13 Oct 2026); dental lab work is Prostheses</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>17278.94</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>18659.88</v>
+        <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45146.24</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>27454.24</v>
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>22166.68</v>
+        <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>13158.04</v>
+        <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23899.96</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>31652.81</v>
+        <v>0</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>19158.99</v>
+        <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>20817.63</v>
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>36588.73</v>
+        <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>39938.75</v>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
         <f>SUM(C6:N6)</f>
@@ -913,44 +913,44 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Implants, crowns, dentures and other implantable devices</t>
+          <t>Implants, abutments, bone graft; crowns, bridges, veneers, onlays, dentures and every other lab-fabricated prosthesis (in-house CAD/CAM materials and external lab invoices)</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>52796</v>
+        <v>70074.94</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>18659.88</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0</v>
+        <v>45146.24</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>27454.24</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>22166.68</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>13158.04</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>23899.96</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0</v>
+        <v>31652.81</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0</v>
+        <v>19158.99</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0</v>
+        <v>20817.63</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>36588.73</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>39938.75</v>
       </c>
       <c r="O9" s="3">
         <f>SUM(C9:N9)</f>
@@ -1613,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1997,12 +1997,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Direct — laboratory (cost centre 09)</t>
+          <t>Direct — prostheses (cost centre 09, in-house CAD/CAM)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>in-house dental laboratory technicians</t>
+          <t>dental technicians making prostheses; routed to the Prosthesis bucket on prosthesis claims (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
@@ -2048,397 +2048,397 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Internal LAB</t>
+          <t>Cost of Goods Sold (M01): Pharmacy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Direct — laboratory</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>in-house dental laboratory materials</t>
+          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1252</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>18259.88</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>21431.24</v>
+        <v>0</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>21431.24</v>
+        <v>0</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>7316.68</v>
+        <v>0</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>13158.04</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>13819.96</v>
+        <v>0</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>20017.81</v>
+        <v>0</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>16858.99</v>
+        <v>0</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>18917.63</v>
+        <v>0</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>15006.23</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>15194.75</v>
+        <v>0</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>181412.45</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>External Lab</t>
+          <t>Cost of Goods Sold: Internal LAB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Direct — laboratory</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>outsourced dental laboratory invoices (expense head)</t>
+          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1870</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>200</v>
+        <v>18259.88</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>16430</v>
+        <v>21431.24</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>4288</v>
+        <v>21431.24</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>7425</v>
+        <v>7316.68</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0</v>
+        <v>13158.04</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>5270</v>
+        <v>13819.96</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>6381</v>
+        <v>20017.81</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>1150</v>
+        <v>16858.99</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>950</v>
+        <v>18917.63</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>10595</v>
+        <v>15006.23</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>12186.25</v>
+        <v>15194.75</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>66745.25</v>
+        <v>181412.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: External LAB</t>
+          <t>Cost of Goods Sold (M01): Prostheses</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Direct — laboratory</t>
+          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>outsourced laboratory invoices booked in cost of goods sold</t>
+          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>68204.94</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>7285</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>1735</v>
+        <v>0</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>7425</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>4810</v>
+        <v>0</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>5254</v>
+        <v>0</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>10987.5</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>12557.75</v>
+        <v>0</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>52354.25</v>
+        <v>68204.94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Laboratory</t>
+          <t>External Lab</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Direct — laboratory</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>in-house lab materials (blocks, blanks, 3D inks, stone, milling tools) + external lab invoices</t>
+          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>15408.94</v>
+        <v>1870</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0</v>
+        <v>16430</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0</v>
+        <v>4288</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0</v>
+        <v>7425</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>5270</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0</v>
+        <v>6381</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0</v>
+        <v>1150</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0</v>
+        <v>10595</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0</v>
+        <v>12186.25</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>15408.94</v>
+        <v>66745.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Pharmacy</t>
+          <t>Cost of Goods Sold: External LAB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pharmacy</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
+          <t>prostheses bought from external laboratories, booked in cost of goods sold</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1252</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0</v>
+        <v>7285</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0</v>
+        <v>1735</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0</v>
+        <v>7425</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0</v>
+        <v>4810</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0</v>
+        <v>5254</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0</v>
+        <v>1150</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0</v>
+        <v>10987.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0</v>
+        <v>12557.75</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>1252</v>
+        <v>52354.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Prostheses</t>
+          <t>Cost of Goods Sold: Consumables -( Dr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Direct — implants</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials</t>
+          <t>clinical consumables issued to the dental surgeries</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>52796</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0</v>
+        <v>67171.58</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0</v>
+        <v>70803.81</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0</v>
+        <v>70803.81</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0</v>
+        <v>63371.43</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0</v>
+        <v>61129.96</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>46785.8</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0</v>
+        <v>67034.7</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0</v>
+        <v>62943.56</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0</v>
+        <v>51591.7</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0</v>
+        <v>39376.22</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0</v>
+        <v>50594.58</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>52796</v>
+        <v>651607.15</v>
       </c>
     </row>
     <row r="13">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -( Dr</t>
+          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2459,63 +2459,63 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — CSSD</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>clinical consumables issued to the dental surgeries</t>
+          <t>sterilisation and vital-signs consumables</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>67171.58</v>
+        <v>3617.35</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>70803.81</v>
+        <v>4867.36</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>70803.81</v>
+        <v>4867.36</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>63371.43</v>
+        <v>4137.43</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>61129.96</v>
+        <v>4094.41</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>46785.8</v>
+        <v>4096.91</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>67034.7</v>
+        <v>4535.04</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>62943.56</v>
+        <v>3033.61</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>51591.7</v>
+        <v>3973.98</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>39376.22</v>
+        <v>5793.45</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>50594.58</v>
+        <v>9800.040000000001</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>651607.15</v>
+        <v>52816.94</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
+          <t>Cost of Goods Sold (M01): MS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2525,91 +2525,91 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Direct — CSSD</t>
+          <t>Direct — dental surgeries / CSSD</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>sterilisation and vital-signs consumables</t>
+          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>31662.75</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>3617.35</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>4137.43</v>
+        <v>0</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>4094.41</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>4096.91</v>
+        <v>0</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>4535.04</v>
+        <v>0</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>3033.61</v>
+        <v>0</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>3973.98</v>
+        <v>0</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>5793.45</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>9800.040000000001</v>
+        <v>0</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>52816.94</v>
+        <v>31662.75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): MS</t>
+          <t>Equipment Maintenanace</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / CSSD</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
+          <t>maintenance of dental chairs and clinical equipment</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>31662.75</v>
+        <v>1000</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0</v>
+        <v>2258.57</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0</v>
+        <v>830</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>0</v>
@@ -2627,159 +2627,159 @@
         <v>0</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0</v>
+        <v>1350</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>31662.75</v>
+        <v>5638.57</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>TB depreciation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Equipment Maintenanace</t>
+          <t>Depreciation: Machinery &amp; Equipment</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — dental surgeries / imaging</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>maintenance of dental chairs and clinical equipment</t>
+          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1000</v>
+        <v>10556.61</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>2258.57</v>
+        <v>10556.61</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>830</v>
+        <v>10556.61</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>1350</v>
+        <v>10556.61</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0</v>
+        <v>10556.61</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>200</v>
+        <v>10556.61</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>5638.57</v>
+        <v>126679.32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Depreciation: Machinery &amp; Equipment</t>
+          <t>Staff Qualification And Education</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>OHF</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / imaging</t>
+          <t>Overhead — HR / IT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>10556.61</v>
+        <v>28462.76</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>10556.61</v>
+        <v>13180.32</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>10556.61</v>
+        <v>43627.94</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>10556.61</v>
+        <v>38711.94</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>10556.61</v>
+        <v>55516.92</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>10556.61</v>
+        <v>155175.22</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>10556.61</v>
+        <v>105124.99</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>10556.61</v>
+        <v>98355.2</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>10556.61</v>
+        <v>80992.27</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>10556.61</v>
+        <v>91500.75999999999</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>10556.61</v>
+        <v>46595.58</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>10556.61</v>
+        <v>132188.09</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>126679.32</v>
+        <v>889431.99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education</t>
+          <t>Salaries &amp; Wages: Indirect /Management</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2789,63 +2789,63 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Overhead — HR / IT</t>
+          <t>Overhead — management</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges</t>
+          <t>clinic management</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>28462.76</v>
+        <v>20000</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>13180.32</v>
+        <v>20000</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>43627.94</v>
+        <v>20000</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>38711.94</v>
+        <v>28000</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>55516.92</v>
+        <v>27000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>155175.22</v>
+        <v>27000</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>105124.99</v>
+        <v>28000</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>98355.2</v>
+        <v>28000</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>80992.27</v>
+        <v>28000</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>91500.75999999999</v>
+        <v>28000</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>46595.58</v>
+        <v>28000</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>132188.09</v>
+        <v>28000</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>889431.99</v>
+        <v>310000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Management</t>
+          <t>Legal &amp; Professional Expenses</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2855,63 +2855,63 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Overhead — management</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>clinic management</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>20000</v>
+        <v>44349.17</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>20000</v>
+        <v>12044.19</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>20000</v>
+        <v>12460.82</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>28000</v>
+        <v>13383.95</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>27000</v>
+        <v>20601.3</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>27000</v>
+        <v>44034.76</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>28000</v>
+        <v>13033.16</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>28000</v>
+        <v>22175.9</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>28000</v>
+        <v>18567.92</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>28000</v>
+        <v>13508.57</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>28000</v>
+        <v>21037.68</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>28000</v>
+        <v>18372.04</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>310000</v>
+        <v>253569.46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses</t>
+          <t>Salaries &amp; Wages: Indirect/RAP</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2921,52 +2921,52 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — reception / patient administration</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees</t>
+          <t>reception and patient-administration staff</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>44349.17</v>
+        <v>11598</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>12044.19</v>
+        <v>12400</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>12460.82</v>
+        <v>12232</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>13383.95</v>
+        <v>10000</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>20601.3</v>
+        <v>14200</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>44034.76</v>
+        <v>13700</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>13033.16</v>
+        <v>13669</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>22175.9</v>
+        <v>14500</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>18567.92</v>
+        <v>15000</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>13508.57</v>
+        <v>21550</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>21037.68</v>
+        <v>21759</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>18372.04</v>
+        <v>22125</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>253569.46</v>
+        <v>182733</v>
       </c>
     </row>
     <row r="21">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/RAP</t>
+          <t>Salaries &amp; Wages: External</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2987,52 +2987,52 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Overhead — reception / patient administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>reception and patient-administration staff</t>
+          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>11598</v>
+        <v>7600</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>12400</v>
+        <v>12690</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>12232</v>
+        <v>11520</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>10000</v>
+        <v>9505</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>14200</v>
+        <v>7800</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>13700</v>
+        <v>9070</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>13669</v>
+        <v>9700</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>14500</v>
+        <v>11596</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>15000</v>
+        <v>16600</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>21550</v>
+        <v>15600</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>21759</v>
+        <v>15600</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>22125</v>
+        <v>15600</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>182733</v>
+        <v>142881</v>
       </c>
     </row>
     <row r="22">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: External</t>
+          <t>Salaries &amp; Wages: Indirect /INS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3053,63 +3053,63 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
+          <t>insurance claims staff</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>7600</v>
+        <v>4400</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>12690</v>
+        <v>5000</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>11520</v>
+        <v>10567</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>9505</v>
+        <v>11500</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>7800</v>
+        <v>12000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>9070</v>
+        <v>10403</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>9700</v>
+        <v>11336</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>11596</v>
+        <v>10871</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>16600</v>
+        <v>11054</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>15600</v>
+        <v>11248</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>15600</v>
+        <v>11234</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>15600</v>
+        <v>11982.5</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>142881</v>
+        <v>121595.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /INS</t>
+          <t>Clinic Rent</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3119,52 +3119,52 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>insurance claims staff</t>
+          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>4400</v>
+        <v>7083.33</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>5000</v>
+        <v>7083.33</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>10567</v>
+        <v>7083.33</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>11500</v>
+        <v>7083.33</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>12000</v>
+        <v>7083.33</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>10403</v>
+        <v>7083.33</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>11336</v>
+        <v>7083.33</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>10871</v>
+        <v>7083.33</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>11054</v>
+        <v>7083.33</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>11248</v>
+        <v>7083.33</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>11234</v>
+        <v>7083.33</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>11982.5</v>
+        <v>7083.33</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>121595.5</v>
+        <v>84999.96000000001</v>
       </c>
     </row>
     <row r="24">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Clinic Rent</t>
+          <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3185,52 +3185,52 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — IT / administration</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
+          <t>software subscriptions, memberships</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>7083.33</v>
+        <v>5585</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>7083.33</v>
+        <v>9203.280000000001</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>7083.33</v>
+        <v>8414.280000000001</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>7083.33</v>
+        <v>2000</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>7083.33</v>
+        <v>6503.7</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>7083.33</v>
+        <v>10028.04</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>7083.33</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>7083.33</v>
+        <v>1842.43</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>7083.33</v>
+        <v>15774.05</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>7083.33</v>
+        <v>6523.81</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>7083.33</v>
+        <v>8884.18</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>7083.33</v>
+        <v>5667.86</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>84999.96000000001</v>
+        <v>80526.17</v>
       </c>
     </row>
     <row r="25">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dues &amp; Subscriptions</t>
+          <t>Finance Charges</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3251,63 +3251,63 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Overhead — IT / administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>software subscriptions, memberships</t>
+          <t>bank and card charges</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>5585</v>
+        <v>6820.88</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>9203.280000000001</v>
+        <v>6684.05</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>8414.280000000001</v>
+        <v>9269.73</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>2000</v>
+        <v>5865.9</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>6503.7</v>
+        <v>5876.86</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>10028.04</v>
+        <v>4410.88</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>99.54000000000001</v>
+        <v>3220.43</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>1842.43</v>
+        <v>4136.27</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>15774.05</v>
+        <v>4080.58</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>6523.81</v>
+        <v>4032.3</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>8884.18</v>
+        <v>4905.68</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>5667.86</v>
+        <v>3702.29</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>80526.17</v>
+        <v>63005.85</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Finance Charges</t>
+          <t>Salaries &amp; Wages: Indirect /Purchase</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3322,58 +3322,58 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>bank and card charges</t>
+          <t>purchasing</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>6820.88</v>
+        <v>5000</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>6684.05</v>
+        <v>5000</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>9269.73</v>
+        <v>5000</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>5865.9</v>
+        <v>5000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>5876.86</v>
+        <v>4458</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>4410.88</v>
+        <v>5000</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>3220.43</v>
+        <v>5000</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>4136.27</v>
+        <v>5000</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>4080.58</v>
+        <v>5000</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>4032.3</v>
+        <v>5000</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>4905.68</v>
+        <v>4758</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>3702.29</v>
+        <v>4958.33</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>63005.85</v>
+        <v>59174.33</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Purchase</t>
+          <t>Utilities Expenses</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3383,52 +3383,52 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>purchasing</t>
+          <t>ADDC electricity/water, Etisalat telephone and internet</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5000</v>
+        <v>4780.25</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>5000</v>
+        <v>4568.37</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>5000</v>
+        <v>4510.14</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>5000</v>
+        <v>4191.56</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>4458</v>
+        <v>8334.92</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>5000</v>
+        <v>4350.26</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>5000</v>
+        <v>4242.75</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>5000</v>
+        <v>4051.47</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>5000</v>
+        <v>4127.37</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>5000</v>
+        <v>4358.95</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>4758</v>
+        <v>4242.9</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>4958.33</v>
+        <v>4322.62</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>59174.33</v>
+        <v>56081.56</v>
       </c>
     </row>
     <row r="28">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Utilities Expenses</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3449,63 +3449,63 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ADDC electricity/water, Etisalat telephone and internet</t>
+          <t>Meta/WhatsApp API, Adobe, promotions</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>4780.25</v>
+        <v>5820.11</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>4568.37</v>
+        <v>2380.86</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>4510.14</v>
+        <v>4382.51</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>4191.56</v>
+        <v>4044.86</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>8334.92</v>
+        <v>4998.58</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>4350.26</v>
+        <v>8392.940000000001</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>4242.75</v>
+        <v>3713.11</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>4051.47</v>
+        <v>5896.89</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>4127.37</v>
+        <v>2707.23</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>4358.95</v>
+        <v>1973.75</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>4242.9</v>
+        <v>8600.299999999999</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>4322.62</v>
+        <v>2478.75</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>56081.56</v>
+        <v>55389.89</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Salaries &amp; Wages: Indirect/Accounts</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3520,58 +3520,58 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Meta/WhatsApp API, Adobe, promotions</t>
+          <t>accounts</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>5820.11</v>
+        <v>4645</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>2380.86</v>
+        <v>3355</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>4382.51</v>
+        <v>4500</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>4044.86</v>
+        <v>4000</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>4998.58</v>
+        <v>3956</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>8392.940000000001</v>
+        <v>4391</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>3713.11</v>
+        <v>4938</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>5896.89</v>
+        <v>3975</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>2707.23</v>
+        <v>4090</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>1973.75</v>
+        <v>4016</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>8600.299999999999</v>
+        <v>4658</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>2478.75</v>
+        <v>4656.25</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>55389.89</v>
+        <v>51180.25</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/Accounts</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3586,47 +3586,47 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>accounts</t>
+          <t>prepaid insurance amortised (staff medical insurance, Daman)</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>4645</v>
+        <v>5939.4</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>3355</v>
+        <v>5974.65</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>4500</v>
+        <v>5974.65</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>4000</v>
+        <v>5974.65</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>3956</v>
+        <v>5995.8</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>4391</v>
+        <v>5995.8</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>4938</v>
+        <v>4564.01</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>3975</v>
+        <v>1833.1</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>4090</v>
+        <v>1974.43</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>4016</v>
+        <v>1974.43</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>4658</v>
+        <v>2038.43</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>4656.25</v>
+        <v>2169.92</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>51180.25</v>
+        <v>50409.27</v>
       </c>
     </row>
     <row r="31">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Repair &amp; Maintenance Expenses</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3647,52 +3647,52 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman)</t>
+          <t>general premises maintenance supplies and works</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5939.4</v>
+        <v>3948.75</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>5974.65</v>
+        <v>701.2</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>5974.65</v>
+        <v>1519</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>5974.65</v>
+        <v>2904.65</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>5995.8</v>
+        <v>418.3</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>5995.8</v>
+        <v>3500</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>4564.01</v>
+        <v>579.13</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>1833.1</v>
+        <v>3615.85</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>1974.43</v>
+        <v>4075.55</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>1974.43</v>
+        <v>4223.2</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>2038.43</v>
+        <v>2824</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>2169.92</v>
+        <v>704.67</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>50409.27</v>
+        <v>29014.3</v>
       </c>
     </row>
     <row r="32">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Repair &amp; Maintenance Expenses</t>
+          <t>Travelling &amp; Transportation</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3713,52 +3713,52 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>general premises maintenance supplies and works</t>
+          <t>taxis, parking, petrol, car wash</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>3948.75</v>
+        <v>1620.78</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>701.2</v>
+        <v>2671.44</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1519</v>
+        <v>1406.51</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>2904.65</v>
+        <v>2252.91</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>418.3</v>
+        <v>2285.53</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>3500</v>
+        <v>1225.52</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>579.13</v>
+        <v>5340.97</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>3615.85</v>
+        <v>1464.2</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>4075.55</v>
+        <v>1523</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>4223.2</v>
+        <v>3348</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>2824</v>
+        <v>2184.07</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>704.67</v>
+        <v>2346.5</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>29014.3</v>
+        <v>27669.43</v>
       </c>
     </row>
     <row r="33">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Travelling &amp; Transportation</t>
+          <t>Fines</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3784,47 +3784,47 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>taxis, parking, petrol, car wash</t>
+          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>1620.78</v>
+        <v>1635</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>2671.44</v>
+        <v>263</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1406.51</v>
+        <v>0</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>2252.91</v>
+        <v>1278</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>2285.53</v>
+        <v>0</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1225.52</v>
+        <v>1031</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>5340.97</v>
+        <v>0</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>1464.2</v>
+        <v>8435.120000000001</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>1523</v>
+        <v>1503</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>3348</v>
+        <v>0</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>2184.07</v>
+        <v>2242.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>2346.5</v>
+        <v>625</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>27669.43</v>
+        <v>17013.03</v>
       </c>
     </row>
     <row r="34">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fines</t>
+          <t>Pantry</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3845,52 +3845,52 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>1635</v>
+        <v>1576.08</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>263</v>
+        <v>1074.12</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0</v>
+        <v>748.9299999999999</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>1278</v>
+        <v>1483.1</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0</v>
+        <v>705.55</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1031</v>
+        <v>1314.1</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0</v>
+        <v>1310.92</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>8435.120000000001</v>
+        <v>1821.61</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>1503</v>
+        <v>1056.15</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0</v>
+        <v>1638.4</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>2242.91</v>
+        <v>1660.35</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>625</v>
+        <v>752.78</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>17013.03</v>
+        <v>15142.09</v>
       </c>
     </row>
     <row r="35">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pantry</t>
+          <t>Other Expenses</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3911,52 +3911,52 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+          <t>courier, flags/badges, miscellaneous</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>1576.08</v>
+        <v>2138.76</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1074.12</v>
+        <v>1089.69</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>748.9299999999999</v>
+        <v>1123.01</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>1483.1</v>
+        <v>3789.07</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>705.55</v>
+        <v>1320.49</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1314.1</v>
+        <v>989.6799999999999</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>1310.92</v>
+        <v>1127.98</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>1821.61</v>
+        <v>1253.75</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>1056.15</v>
+        <v>508.94</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>1638.4</v>
+        <v>264.83</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>1660.35</v>
+        <v>316.45</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>752.78</v>
+        <v>88.53</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>15142.09</v>
+        <v>14011.18</v>
       </c>
     </row>
     <row r="36">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3982,47 +3982,47 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>courier, flags/badges, miscellaneous</t>
+          <t>stationery, printer ink, newspapers</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>2138.76</v>
+        <v>783.13</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1089.69</v>
+        <v>449.05</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1123.01</v>
+        <v>373</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>3789.07</v>
+        <v>1618.98</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>1320.49</v>
+        <v>404.77</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>989.6799999999999</v>
+        <v>1228.67</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>1127.98</v>
+        <v>340.61</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>1253.75</v>
+        <v>481.01</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>508.94</v>
+        <v>1156.65</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>264.83</v>
+        <v>440.57</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>316.45</v>
+        <v>237.4</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>88.53</v>
+        <v>375.55</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>14011.18</v>
+        <v>7889.39</v>
       </c>
     </row>
     <row r="37">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Claim Rejection</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4043,63 +4043,63 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>stationery, printer ink, newspapers</t>
+          <t>written-off rejected claims</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>783.13</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>449.05</v>
+        <v>0</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>373</v>
+        <v>844.2</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>1618.98</v>
+        <v>0</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>404.77</v>
+        <v>0</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1228.67</v>
+        <v>245</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>340.61</v>
+        <v>0</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>481.01</v>
+        <v>0</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>1156.65</v>
+        <v>1005</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>440.57</v>
+        <v>-32</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>237.4</v>
+        <v>1235</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>375.55</v>
+        <v>105</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>7889.39</v>
+        <v>3402.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Claim Rejection</t>
+          <t>Cost of Goods Sold (M01): OHF</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4109,22 +4109,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>written-off rejected claims</t>
+          <t>pantry and stationery issued from stock</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>0</v>
+        <v>1007.8</v>
       </c>
       <c r="G38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>844.2</v>
+        <v>0</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>0</v>
@@ -4133,7 +4133,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="L38" s="3" t="n">
         <v>0</v>
@@ -4142,30 +4142,30 @@
         <v>0</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>1005</v>
+        <v>0</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>-32</v>
+        <v>0</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>1235</v>
+        <v>0</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>3402.2</v>
+        <v>1007.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): OHF</t>
+          <t>Salaries &amp; Wages: Indirect it</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4175,16 +4175,16 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — IT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>pantry and stationery issued from stock</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1007.8</v>
+        <v>0</v>
       </c>
       <c r="G39" s="3" t="n">
         <v>0</v>
@@ -4220,7 +4220,7 @@
         <v>0</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>1007.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect it</t>
+          <t>Salaries &amp; Wages: Indirect/ Hr</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4241,12 +4241,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Overhead — IT</t>
+          <t>Overhead — HR</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F40" s="3" t="n">
@@ -4292,221 +4292,205 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>TB depreciation</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+          <t>Depreciation: furniture, office equipment, computers, software</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>OHDepreciation</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Overhead — HR</t>
+          <t>Overhead — facility / IT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>0</v>
+        <v>2524.8</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>0</v>
+        <v>30297.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Depreciation: furniture, office equipment, computers, software</t>
+          <t>Third Party &amp; Professional Services</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>OHDepreciation</t>
+          <t>OHC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Overhead — facility / IT</t>
+          <t>Overhead — shared services</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+          <t>MySmyle Company EMR subscription, management consultancy and IT services (25,000/month) + Calibrate/Platform Technologies: services charged by a sister company = corporate/shared-services overhead</t>
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>2524.8</v>
+        <v>8317</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>2524.8</v>
+        <v>37300</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>2524.8</v>
+        <v>62270</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>2524.8</v>
+        <v>66480.95</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>2524.8</v>
+        <v>2500</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>2524.8</v>
+        <v>37375.73</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>2524.8</v>
+        <v>25000</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>2524.8</v>
+        <v>27500</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>2524.8</v>
+        <v>28000</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>2524.8</v>
+        <v>25500</v>
       </c>
       <c r="P42" s="3" t="n">
-        <v>2524.8</v>
+        <v>25000</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>2524.8</v>
+        <v>25104.5</v>
       </c>
       <c r="R42" s="3" t="n">
-        <v>30297.6</v>
+        <v>370348.18</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Monthly sheet</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Third Party &amp; Professional Services</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>OHC</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Overhead — shared services</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>MySmyle Company EMR subscription, management consultancy and IT services (25,000/month) + Calibrate/Platform Technologies: services charged by a sister company = corporate/shared-services overhead</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>8317</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>37300</v>
-      </c>
-      <c r="H43" s="3" t="n">
-        <v>62270</v>
-      </c>
-      <c r="I43" s="3" t="n">
-        <v>66480.95</v>
-      </c>
-      <c r="J43" s="3" t="n">
-        <v>2500</v>
-      </c>
-      <c r="K43" s="3" t="n">
-        <v>37375.73</v>
-      </c>
-      <c r="L43" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="M43" s="3" t="n">
-        <v>27500</v>
-      </c>
-      <c r="N43" s="3" t="n">
-        <v>28000</v>
-      </c>
-      <c r="O43" s="3" t="n">
-        <v>25500</v>
-      </c>
-      <c r="P43" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="Q43" s="3" t="n">
-        <v>25104.5</v>
-      </c>
-      <c r="R43" s="3" t="n">
-        <v>370348.18</v>
-      </c>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="3" t="n"/>
-      <c r="K44" s="3" t="n"/>
-      <c r="L44" s="3" t="n"/>
-      <c r="M44" s="3" t="n"/>
-      <c r="N44" s="3" t="n"/>
-      <c r="O44" s="3" t="n"/>
-      <c r="P44" s="3" t="n"/>
-      <c r="Q44" s="3" t="n"/>
-      <c r="R44" s="3" t="n"/>
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL mapped</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="5" t="n">
+        <v>511302.3</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>532341.65</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>606868.87</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>518123.67</v>
+      </c>
+      <c r="J44" s="5" t="n">
+        <v>488066.69</v>
+      </c>
+      <c r="K44" s="5" t="n">
+        <v>616494.08</v>
+      </c>
+      <c r="L44" s="5" t="n">
+        <v>480166.81</v>
+      </c>
+      <c r="M44" s="5" t="n">
+        <v>526990.09</v>
+      </c>
+      <c r="N44" s="5" t="n">
+        <v>509542.04</v>
+      </c>
+      <c r="O44" s="5" t="n">
+        <v>546725.96</v>
+      </c>
+      <c r="P44" s="5" t="n">
+        <v>493746.03</v>
+      </c>
+      <c r="Q44" s="5" t="n">
+        <v>623033.72</v>
+      </c>
+      <c r="R44" s="5" t="n">
+        <v>6453401.91</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr"/>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>TOTAL mapped</t>
+          <t>Ledger (locked)</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr"/>
@@ -4528,77 +4512,27 @@
         <v>488066.69</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>616494.08</v>
+        <v>616494.09</v>
       </c>
       <c r="L45" s="5" t="n">
-        <v>480166.81</v>
+        <v>480166.82</v>
       </c>
       <c r="M45" s="5" t="n">
-        <v>526990.09</v>
+        <v>526990.1</v>
       </c>
       <c r="N45" s="5" t="n">
-        <v>509542.04</v>
+        <v>509542.05</v>
       </c>
       <c r="O45" s="5" t="n">
-        <v>546725.96</v>
+        <v>546725.98</v>
       </c>
       <c r="P45" s="5" t="n">
         <v>493746.03</v>
       </c>
       <c r="Q45" s="5" t="n">
-        <v>623033.72</v>
+        <v>623033.73</v>
       </c>
       <c r="R45" s="5" t="n">
-        <v>6453401.91</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr"/>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Ledger (locked)</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="5" t="n">
-        <v>511302.3</v>
-      </c>
-      <c r="G46" s="5" t="n">
-        <v>532341.65</v>
-      </c>
-      <c r="H46" s="5" t="n">
-        <v>606868.87</v>
-      </c>
-      <c r="I46" s="5" t="n">
-        <v>518123.67</v>
-      </c>
-      <c r="J46" s="5" t="n">
-        <v>488066.69</v>
-      </c>
-      <c r="K46" s="5" t="n">
-        <v>616494.09</v>
-      </c>
-      <c r="L46" s="5" t="n">
-        <v>480166.82</v>
-      </c>
-      <c r="M46" s="5" t="n">
-        <v>526990.1</v>
-      </c>
-      <c r="N46" s="5" t="n">
-        <v>509542.05</v>
-      </c>
-      <c r="O46" s="5" t="n">
-        <v>546725.98</v>
-      </c>
-      <c r="P46" s="5" t="n">
-        <v>493746.03</v>
-      </c>
-      <c r="Q46" s="5" t="n">
-        <v>623033.73</v>
-      </c>
-      <c r="R46" s="5" t="n">
         <v>6453401.98</v>
       </c>
     </row>
@@ -4643,7 +4577,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q3. Prostheses, Pharmacy and Imaging cost types are 0: implants, anaesthetics and imaging sensors are bought inside 'Consumables' (MS). If the purchase ledger can separate them, they should move to those cost types.</t>
+          <t>Q3. Laboratory cost type is 0 by ruling (13 Oct 2026): the clinic has no laboratory; in-house CAD/CAM materials, external lab invoices and implants are Prostheses, and the dental technicians' pay (SWAllied) is routed to the Prosthesis bucket. Pharmacy and Imaging consumables are split from stock only for the months with a stock-movement sheet; the other months keep them inside MS until the sheets arrive.</t>
         </is>
       </c>
     </row>
@@ -4814,238 +4748,238 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           130.00</t>
+          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   05- Medical Electronic Devices (Restorative, Perio, Endo, Implants, Ortho…)    5,500.00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,889.75</t>
+          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo, Implants,Ortho…)       83.33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           03- Dental Blanks                                   1,875.00</t>
+          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   345.28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              5,000.00</t>
+          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,993.20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   58.19</t>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,477.50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        985.00</t>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,007.00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessories     1,601.00</t>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        540.65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   05- Medical Electronic Devices (Restorative, Perio, Endo, Implants, Ortho…)    5,500.00</t>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   338.00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo, Implants,Ortho…)       83.33</t>
+          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          806.00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   345.28</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,552.50</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,993.20</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            756.62</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,477.50</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      4,441.00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,007.00</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,630.33</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        540.65</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     710.82</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   338.00</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   690.50</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          806.00</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,700.00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,552.50</t>
+          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            90.00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            756.62</t>
+          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   847.80</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      4,441.00</t>
+          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  160.00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,630.33</t>
+          <t>Movement Jan 2025: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                682.00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     710.82</t>
+          <t>Movement Jan 2025: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         570.00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   690.50</t>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               27,500.00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,700.00</t>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           3,699.00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            90.00</t>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       6,652.00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   847.80</t>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               960.00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  160.00</t>
+          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             13,985.00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                682.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           130.00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         570.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,889.75</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               27,500.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   1,875.00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           3,699.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              5,000.00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       6,652.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   58.19</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               960.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        985.00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             13,985.00</t>
+          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessories     1,601.00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Laboratory  External LAB (P&amp;L line, not stock)                                            1,870.00</t>
+          <t>Movement Jan 2025: Prostheses  External LAB invoices (P&amp;L line, not stock)                                        1,870.00</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6175,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>laboratory technicians / (laboratory technicians + CSSD technicians), Salary sheet; drives the Laboratory bucket</t>
+          <t>dental technicians / (dental technicians + CSSD technicians), Salary sheet; the engine pre-assigns this share of SWAllied to the Prosthesis bucket on the prosthesis-coded claims (ruling 13 Oct 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruling: staff on-costs split by monthly salary share into SWDoc/SWNurs/SWAllied/OHF; refill ledger map; re-run January
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -553,40 +553,40 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>25100</v>
+        <v>31532.24</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>25952</v>
+        <v>28267.94</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>25607</v>
+        <v>30636.78</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>25486</v>
+        <v>31474.11</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>29050</v>
+        <v>37720.38</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>29143.33</v>
+        <v>53560.11</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>26699.8</v>
+        <v>41977.45</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>29433</v>
+        <v>45741.97</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>20417</v>
+        <v>29312.81</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>29125</v>
+        <v>40078.65</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>29266.13</v>
+        <v>36879.04</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>29416.67</v>
+        <v>44482.71</v>
       </c>
       <c r="O2" s="3">
         <f>SUM(C2:N2)</f>
@@ -605,40 +605,40 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>171870</v>
+        <v>215914.15</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>225878.31</v>
+        <v>246035.58</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>206907</v>
+        <v>247548.14</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>136987</v>
+        <v>169173.03</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>152254</v>
+        <v>197696.32</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>132942</v>
+        <v>244323.08</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>107479</v>
+        <v>168978.6</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>102568</v>
+        <v>159401.46</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>122528</v>
+        <v>175914.16</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>162693</v>
+        <v>223880.42</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>129357.35</v>
+        <v>163006.68</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>166275.01</v>
+        <v>251434.38</v>
       </c>
       <c r="O3" s="3">
         <f>SUM(C3:N3)</f>
@@ -657,40 +657,40 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14150</v>
+        <v>17776.15</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>12610</v>
+        <v>13735.31</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12629</v>
+        <v>15109.63</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>9545</v>
+        <v>11787.67</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12045.69</v>
+        <v>15640.89</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>7000</v>
+        <v>12864.73</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>10700</v>
+        <v>16822.55</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>14797</v>
+        <v>22996.09</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>14500</v>
+        <v>20817.73</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>12340.34</v>
+        <v>16981.43</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>15185.48</v>
+        <v>19135.63</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>20317.75</v>
+        <v>30723.69</v>
       </c>
       <c r="O4" s="3">
         <f>SUM(C4:N4)</f>
@@ -1177,40 +1177,40 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>174794.2</v>
+        <v>120691.66</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>125812.55</v>
+        <v>102214.03</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>165557.05</v>
+        <v>117405.5</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>162587.9</v>
+        <v>122171.09</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>189460.05</v>
+        <v>131752.15</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>318569.21</v>
+        <v>176906.62</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>222423.94</v>
+        <v>139524.14</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>236388.14</v>
+        <v>155046.62</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>225879.48</v>
+        <v>157279.78</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>226252.92</v>
+        <v>149470.76</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>200097.26</v>
+        <v>154884.87</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>268305.02</v>
+        <v>157673.67</v>
       </c>
       <c r="O14" s="3">
         <f>SUM(C14:N14)</f>
@@ -1613,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1850,215 +1850,215 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Direct Dr</t>
+          <t>Staff Qualification And Education: on-cost → SWNurs</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SWDoc</t>
+          <t>SWNurs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — dental surgeries (nurses' on-costs)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>dentists, oral surgeon, orthodontist (Salary sheet 'Direct Dr')</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>171870</v>
+        <v>2782.39</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>225878.31</v>
+        <v>1102.71</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>206907</v>
+        <v>3755.96</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>136987</v>
+        <v>4279.98</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>152254</v>
+        <v>6325.48</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>132942</v>
+        <v>19698.3</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>107479</v>
+        <v>13505.88</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>102568</v>
+        <v>13841.6</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>122528</v>
+        <v>7496.38</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>162693</v>
+        <v>9727.110000000001</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>129357.35</v>
+        <v>5583.83</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>166275.01</v>
+        <v>13514.45</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>1817738.67</v>
+        <v>101614.07</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Cssd</t>
+          <t>Legal &amp; Professional Expenses: on-cost → SWNurs</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SWAllied</t>
+          <t>SWNurs</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Direct — CSSD (cost centre 07)</t>
+          <t>Direct — dental surgeries (nurses' on-costs)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sterilisation technicians</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>7000</v>
+        <v>3069.24</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>7000</v>
+        <v>713.37</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>7000</v>
+        <v>759.46</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>6500</v>
+        <v>1047.57</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>7000</v>
+        <v>1661.75</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>7000</v>
+        <v>3957.36</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>7000</v>
+        <v>1185.41</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>7000</v>
+        <v>2209.4</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>7500</v>
+        <v>1216.68</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>7500</v>
+        <v>1016.65</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>7500</v>
+        <v>1784.8</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>8000</v>
+        <v>1329.74</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>86000</v>
+        <v>19951.43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/LAB</t>
+          <t>Insurance: on-cost → SWNurs</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SWAllied</t>
+          <t>SWNurs</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Direct — prostheses (cost centre 09, in-house CAD/CAM)</t>
+          <t>Direct — dental surgeries (nurses' on-costs)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>dental technicians making prostheses; routed to the Prosthesis bucket on prosthesis claims (ruling 13 Oct 2026)</t>
+          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>7150</v>
+        <v>580.61</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>5610</v>
+        <v>499.86</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>5629</v>
+        <v>514.36</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>3045</v>
+        <v>660.5599999999999</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>5045.69</v>
+        <v>683.15</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>761.12</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3700</v>
+        <v>586.36</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>7797</v>
+        <v>257.97</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>7000</v>
+        <v>182.75</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>4840.34</v>
+        <v>209.89</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>7685.48</v>
+        <v>244.28</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>12317.75</v>
+        <v>221.85</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>69820.25999999999</v>
+        <v>5402.76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Pharmacy</t>
+          <t>Salaries &amp; Wages: Direct Dr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pharmacy</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2068,179 +2068,179 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
+          <t>dentists, oral surgeon, orthodontist (Salary sheet 'Direct Dr')</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1252</v>
+        <v>171870</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0</v>
+        <v>225878.31</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0</v>
+        <v>206907</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0</v>
+        <v>136987</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0</v>
+        <v>152254</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0</v>
+        <v>132942</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>0</v>
+        <v>107479</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0</v>
+        <v>102568</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0</v>
+        <v>122528</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0</v>
+        <v>162693</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0</v>
+        <v>129357.35</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0</v>
+        <v>166275.01</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>1252</v>
+        <v>1817738.67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Internal LAB</t>
+          <t>Staff Qualification And Education: on-cost → SWDoc</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — dental surgeries (dentists' on-costs)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>19052.18</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>18259.88</v>
+        <v>9597.66</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>21431.24</v>
+        <v>30348.52</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>21431.24</v>
+        <v>23004.85</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>7316.68</v>
+        <v>33152.46</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>13158.04</v>
+        <v>89856.97</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>13819.96</v>
+        <v>54367.39</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>20017.81</v>
+        <v>48235.17</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>16858.99</v>
+        <v>44987.84</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>18917.63</v>
+        <v>54335.9</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>15006.23</v>
+        <v>24680.75</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>15194.75</v>
+        <v>76389.19</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>181412.45</v>
+        <v>508008.88</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Prostheses</t>
+          <t>Legal &amp; Professional Expenses: on-cost → SWDoc</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
+          <t>Direct — dental surgeries (dentists' on-costs)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>68204.94</v>
+        <v>21016.31</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0</v>
+        <v>6208.98</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0</v>
+        <v>6136.53</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0</v>
+        <v>5630.7</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0</v>
+        <v>8709.41</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0</v>
+        <v>18052.14</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0</v>
+        <v>4771.84</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0</v>
+        <v>7699.3</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0</v>
+        <v>7301.61</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0</v>
+        <v>5679.04</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0</v>
+        <v>7888.87</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>0</v>
+        <v>7516.23</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>68204.94</v>
+        <v>106610.96</v>
       </c>
     </row>
     <row r="10">
@@ -2251,326 +2251,326 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>External Lab</t>
+          <t>Insurance: on-cost → SWDoc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — dental surgeries (dentists' on-costs)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
+          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>1870</v>
+        <v>3975.66</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>200</v>
+        <v>4350.63</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>16430</v>
+        <v>4156.09</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>4288</v>
+        <v>3550.48</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>7425</v>
+        <v>3580.45</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0</v>
+        <v>3471.97</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>5270</v>
+        <v>2360.37</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>6381</v>
+        <v>898.99</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>1150</v>
+        <v>1096.71</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>950</v>
+        <v>1172.48</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>10595</v>
+        <v>1079.71</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>12186.25</v>
+        <v>1253.95</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>66745.25</v>
+        <v>30947.49</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: External LAB</t>
+          <t>Salaries &amp; Wages: Cssd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — CSSD (cost centre 07)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>prostheses bought from external laboratories, booked in cost of goods sold</t>
+          <t>sterilisation technicians</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>7000</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>200</v>
+        <v>7000</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>7285</v>
+        <v>7000</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>1735</v>
+        <v>6500</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>7425</v>
+        <v>7000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
+        <v>7000</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>4810</v>
+        <v>7000</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>5254</v>
+        <v>7000</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>1150</v>
+        <v>7500</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>950</v>
+        <v>7500</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>10987.5</v>
+        <v>7500</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>12557.75</v>
+        <v>8000</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>52354.25</v>
+        <v>86000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -( Dr</t>
+          <t>Salaries &amp; Wages: Indirect/LAB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — prostheses (cost centre 09, in-house CAD/CAM)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>clinical consumables issued to the dental surgeries</t>
+          <t>dental technicians making prostheses; routed to the Prosthesis bucket on prosthesis claims (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>7150</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>67171.58</v>
+        <v>5610</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>70803.81</v>
+        <v>5629</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>70803.81</v>
+        <v>3045</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>63371.43</v>
+        <v>5045.69</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>61129.96</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>46785.8</v>
+        <v>3700</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>67034.7</v>
+        <v>7797</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>62943.56</v>
+        <v>7000</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>51591.7</v>
+        <v>4840.34</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>39376.22</v>
+        <v>7685.48</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>50594.58</v>
+        <v>12317.75</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>651607.15</v>
+        <v>69820.25999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
+          <t>Staff Qualification And Education: on-cost → SWAllied</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Direct — CSSD</t>
+          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sterilisation and vital-signs consumables</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>1568.56</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>3617.35</v>
+        <v>535.8</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>4867.36</v>
+        <v>1852.39</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>4867.36</v>
+        <v>1602.94</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>4137.43</v>
+        <v>2622.88</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>4094.41</v>
+        <v>4731.38</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>4096.91</v>
+        <v>5412.51</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>4535.04</v>
+        <v>6958.66</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>3033.61</v>
+        <v>5323.87</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>3973.98</v>
+        <v>4121.4</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>5793.45</v>
+        <v>2897.31</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>9800.040000000001</v>
+        <v>9334.27</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>52816.94</v>
+        <v>46961.97</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): MS</t>
+          <t>Legal &amp; Professional Expenses: on-cost → SWAllied</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / CSSD</t>
+          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31662.75</v>
+        <v>1730.27</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>346.63</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0</v>
+        <v>374.56</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0</v>
+        <v>392.34</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0</v>
+        <v>689.05</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0</v>
+        <v>950.53</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0</v>
+        <v>475.06</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>1110.74</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0</v>
+        <v>864.0700000000001</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0</v>
+        <v>430.76</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0</v>
+        <v>926.09</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0</v>
+        <v>918.4400000000001</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>31662.75</v>
+        <v>9208.540000000001</v>
       </c>
     </row>
     <row r="15">
@@ -2581,260 +2581,260 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Equipment Maintenanace</t>
+          <t>Insurance: on-cost → SWAllied</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>maintenance of dental chairs and clinical equipment</t>
+          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1000</v>
+        <v>327.32</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>2258.57</v>
+        <v>242.88</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0</v>
+        <v>253.68</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>830</v>
+        <v>247.39</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0</v>
+        <v>283.27</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
+        <v>182.82</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0</v>
+        <v>234.98</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>129.69</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0</v>
+        <v>129.79</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>1350</v>
+        <v>88.93000000000001</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>0</v>
+        <v>126.75</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>200</v>
+        <v>153.23</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>5638.57</v>
+        <v>2400.73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Depreciation: Machinery &amp; Equipment</t>
+          <t>Cost of Goods Sold (M01): Pharmacy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / imaging</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
+          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>10556.61</v>
+        <v>1252</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>126679.32</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education</t>
+          <t>Cost of Goods Sold: Internal LAB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Overhead — HR / IT</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges</t>
+          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28462.76</v>
+        <v>0</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>13180.32</v>
+        <v>18259.88</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>43627.94</v>
+        <v>21431.24</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>38711.94</v>
+        <v>21431.24</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>55516.92</v>
+        <v>7316.68</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>155175.22</v>
+        <v>13158.04</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>105124.99</v>
+        <v>13819.96</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>98355.2</v>
+        <v>20017.81</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>80992.27</v>
+        <v>16858.99</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>91500.75999999999</v>
+        <v>18917.63</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>46595.58</v>
+        <v>15006.23</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>132188.09</v>
+        <v>15194.75</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>889431.99</v>
+        <v>181412.45</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Management</t>
+          <t>Cost of Goods Sold (M01): Prostheses</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Overhead — management</t>
+          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>clinic management</t>
+          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>20000</v>
+        <v>68204.94</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>310000</v>
+        <v>68204.94</v>
       </c>
     </row>
     <row r="19">
@@ -2845,326 +2845,326 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses</t>
+          <t>External Lab</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees</t>
+          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>44349.17</v>
+        <v>1870</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>12044.19</v>
+        <v>200</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>12460.82</v>
+        <v>16430</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>13383.95</v>
+        <v>4288</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>20601.3</v>
+        <v>7425</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>44034.76</v>
+        <v>0</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>13033.16</v>
+        <v>5270</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>22175.9</v>
+        <v>6381</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>18567.92</v>
+        <v>1150</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>13508.57</v>
+        <v>950</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>21037.68</v>
+        <v>10595</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>18372.04</v>
+        <v>12186.25</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>253569.46</v>
+        <v>66745.25</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/RAP</t>
+          <t>Cost of Goods Sold: External LAB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Overhead — reception / patient administration</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>reception and patient-administration staff</t>
+          <t>prostheses bought from external laboratories, booked in cost of goods sold</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>11598</v>
+        <v>0</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>12400</v>
+        <v>200</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>12232</v>
+        <v>7285</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>10000</v>
+        <v>1735</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>14200</v>
+        <v>7425</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>13700</v>
+        <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>13669</v>
+        <v>4810</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>14500</v>
+        <v>5254</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>15000</v>
+        <v>1150</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>21550</v>
+        <v>950</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>21759</v>
+        <v>10987.5</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>22125</v>
+        <v>12557.75</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>182733</v>
+        <v>52354.25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: External</t>
+          <t>Cost of Goods Sold: Consumables -( Dr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
+          <t>clinical consumables issued to the dental surgeries</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>7600</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>12690</v>
+        <v>67171.58</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>11520</v>
+        <v>70803.81</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>9505</v>
+        <v>70803.81</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>7800</v>
+        <v>63371.43</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>9070</v>
+        <v>61129.96</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>9700</v>
+        <v>46785.8</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>11596</v>
+        <v>67034.7</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>16600</v>
+        <v>62943.56</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>15600</v>
+        <v>51591.7</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>15600</v>
+        <v>39376.22</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>15600</v>
+        <v>50594.58</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>142881</v>
+        <v>651607.15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /INS</t>
+          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Direct — CSSD</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>insurance claims staff</t>
+          <t>sterilisation and vital-signs consumables</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>5000</v>
+        <v>3617.35</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>10567</v>
+        <v>4867.36</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>11500</v>
+        <v>4867.36</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>12000</v>
+        <v>4137.43</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>10403</v>
+        <v>4094.41</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>11336</v>
+        <v>4096.91</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>10871</v>
+        <v>4535.04</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>11054</v>
+        <v>3033.61</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>11248</v>
+        <v>3973.98</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>11234</v>
+        <v>5793.45</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>11982.5</v>
+        <v>9800.040000000001</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>121595.5</v>
+        <v>52816.94</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Clinic Rent</t>
+          <t>Cost of Goods Sold (M01): MS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Direct — dental surgeries / CSSD</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
+          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>7083.33</v>
+        <v>31662.75</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>7083.33</v>
+        <v>0</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>84999.96000000001</v>
+        <v>31662.75</v>
       </c>
     </row>
     <row r="24">
@@ -3175,128 +3175,128 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dues &amp; Subscriptions</t>
+          <t>Equipment Maintenanace</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Overhead — IT / administration</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>software subscriptions, memberships</t>
+          <t>maintenance of dental chairs and clinical equipment</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5585</v>
+        <v>1000</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>9203.280000000001</v>
+        <v>2258.57</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>8414.280000000001</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>2000</v>
+        <v>830</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>6503.7</v>
+        <v>0</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>10028.04</v>
+        <v>0</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>99.54000000000001</v>
+        <v>0</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>1842.43</v>
+        <v>0</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>15774.05</v>
+        <v>0</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>6523.81</v>
+        <v>1350</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>8884.18</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>5667.86</v>
+        <v>200</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>80526.17</v>
+        <v>5638.57</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>TB depreciation</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Finance Charges</t>
+          <t>Depreciation: Machinery &amp; Equipment</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Direct — dental surgeries / imaging</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bank and card charges</t>
+          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>6820.88</v>
+        <v>10556.61</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6684.05</v>
+        <v>10556.61</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>9269.73</v>
+        <v>10556.61</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>5865.9</v>
+        <v>10556.61</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>5876.86</v>
+        <v>10556.61</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>4410.88</v>
+        <v>10556.61</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>3220.43</v>
+        <v>10556.61</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>4136.27</v>
+        <v>10556.61</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>4080.58</v>
+        <v>10556.61</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>4032.3</v>
+        <v>10556.61</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>4905.68</v>
+        <v>10556.61</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>3702.29</v>
+        <v>10556.61</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>63005.85</v>
+        <v>126679.32</v>
       </c>
     </row>
     <row r="26">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Purchase</t>
+          <t>Salaries &amp; Wages: Indirect /Management</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3317,52 +3317,52 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — management</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>purchasing</t>
+          <t>clinic management</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>5000</v>
+        <v>28000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>4458</v>
+        <v>27000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>5000</v>
+        <v>27000</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>5000</v>
+        <v>28000</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>5000</v>
+        <v>28000</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>5000</v>
+        <v>28000</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>5000</v>
+        <v>28000</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>4758</v>
+        <v>28000</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>4958.33</v>
+        <v>28000</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>59174.33</v>
+        <v>310000</v>
       </c>
     </row>
     <row r="27">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Utilities Expenses</t>
+          <t>Staff Qualification And Education: on-cost → OHF</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3383,63 +3383,63 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — back-office staff on-costs</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ADDC electricity/water, Etisalat telephone and internet</t>
+          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>4780.25</v>
+        <v>5059.63</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>4568.37</v>
+        <v>1944.15</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>4510.14</v>
+        <v>7671.07</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>4191.56</v>
+        <v>9824.17</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>8334.92</v>
+        <v>13416.1</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>4350.26</v>
+        <v>40888.57</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>4242.75</v>
+        <v>31839.21</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>4051.47</v>
+        <v>29319.77</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>4127.37</v>
+        <v>23184.18</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>4358.95</v>
+        <v>23316.35</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>4242.9</v>
+        <v>13433.69</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>4322.62</v>
+        <v>32950.18</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>56081.56</v>
+        <v>232847.07</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Salaries &amp; Wages: Indirect/RAP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3449,52 +3449,52 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — reception / patient administration</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Meta/WhatsApp API, Adobe, promotions</t>
+          <t>reception and patient-administration staff</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>5820.11</v>
+        <v>11598</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>2380.86</v>
+        <v>12400</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>4382.51</v>
+        <v>12232</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>4044.86</v>
+        <v>10000</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>4998.58</v>
+        <v>14200</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>8392.940000000001</v>
+        <v>13700</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>3713.11</v>
+        <v>13669</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>5896.89</v>
+        <v>14500</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>2707.23</v>
+        <v>15000</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>1973.75</v>
+        <v>21550</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>8600.299999999999</v>
+        <v>21759</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>2478.75</v>
+        <v>22125</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>55389.89</v>
+        <v>182733</v>
       </c>
     </row>
     <row r="29">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/Accounts</t>
+          <t>Salaries &amp; Wages: External</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3520,58 +3520,58 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>accounts</t>
+          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>4645</v>
+        <v>7600</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>3355</v>
+        <v>12690</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>4500</v>
+        <v>11520</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>4000</v>
+        <v>9505</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>3956</v>
+        <v>7800</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>4391</v>
+        <v>9070</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>4938</v>
+        <v>9700</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>3975</v>
+        <v>11596</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>4090</v>
+        <v>16600</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>4016</v>
+        <v>15600</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>4658</v>
+        <v>15600</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>4656.25</v>
+        <v>15600</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>51180.25</v>
+        <v>142881</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Salaries &amp; Wages: Indirect /INS</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3581,52 +3581,52 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman)</t>
+          <t>insurance claims staff</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5939.4</v>
+        <v>4400</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>5974.65</v>
+        <v>5000</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>5974.65</v>
+        <v>10567</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>5974.65</v>
+        <v>11500</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>5995.8</v>
+        <v>12000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>5995.8</v>
+        <v>10403</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>4564.01</v>
+        <v>11336</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>1833.1</v>
+        <v>10871</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>1974.43</v>
+        <v>11054</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>1974.43</v>
+        <v>11248</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>2038.43</v>
+        <v>11234</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>2169.92</v>
+        <v>11982.5</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>50409.27</v>
+        <v>121595.5</v>
       </c>
     </row>
     <row r="31">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Repair &amp; Maintenance Expenses</t>
+          <t>Clinic Rent</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3652,47 +3652,47 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>general premises maintenance supplies and works</t>
+          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>3948.75</v>
+        <v>7083.33</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>701.2</v>
+        <v>7083.33</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1519</v>
+        <v>7083.33</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>2904.65</v>
+        <v>7083.33</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>418.3</v>
+        <v>7083.33</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>3500</v>
+        <v>7083.33</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>579.13</v>
+        <v>7083.33</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>3615.85</v>
+        <v>7083.33</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>4075.55</v>
+        <v>7083.33</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>4223.2</v>
+        <v>7083.33</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>2824</v>
+        <v>7083.33</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>704.67</v>
+        <v>7083.33</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>29014.3</v>
+        <v>84999.96000000001</v>
       </c>
     </row>
     <row r="32">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Travelling &amp; Transportation</t>
+          <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3713,52 +3713,52 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — IT / administration</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>taxis, parking, petrol, car wash</t>
+          <t>software subscriptions, memberships</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>1620.78</v>
+        <v>5585</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2671.44</v>
+        <v>9203.280000000001</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1406.51</v>
+        <v>8414.280000000001</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>2252.91</v>
+        <v>2000</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>2285.53</v>
+        <v>6503.7</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1225.52</v>
+        <v>10028.04</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>5340.97</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>1464.2</v>
+        <v>1842.43</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>1523</v>
+        <v>15774.05</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>3348</v>
+        <v>6523.81</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>2184.07</v>
+        <v>8884.18</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>2346.5</v>
+        <v>5667.86</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>27669.43</v>
+        <v>80526.17</v>
       </c>
     </row>
     <row r="33">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fines</t>
+          <t>Legal &amp; Professional Expenses: non-on-cost part</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3784,47 +3784,47 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees (facility licences, accreditation, trade licence)</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>1635</v>
+        <v>12952.11</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>263</v>
+        <v>3517.49</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0</v>
+        <v>3639.16</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>1278</v>
+        <v>3908.76</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0</v>
+        <v>6016.58</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1031</v>
+        <v>12860.28</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0</v>
+        <v>3806.31</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>8435.120000000001</v>
+        <v>6476.44</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>1503</v>
+        <v>5422.73</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0</v>
+        <v>3945.16</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>2242.91</v>
+        <v>6144.02</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>625</v>
+        <v>5365.53</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>17013.03</v>
+        <v>74054.57000000001</v>
       </c>
     </row>
     <row r="34">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pantry</t>
+          <t>Finance Charges</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3845,63 +3845,63 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+          <t>bank and card charges</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>1576.08</v>
+        <v>6820.88</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>1074.12</v>
+        <v>6684.05</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>748.9299999999999</v>
+        <v>9269.73</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>1483.1</v>
+        <v>5865.9</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>705.55</v>
+        <v>5876.86</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1314.1</v>
+        <v>4410.88</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>1310.92</v>
+        <v>3220.43</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>1821.61</v>
+        <v>4136.27</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>1056.15</v>
+        <v>4080.58</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>1638.4</v>
+        <v>4032.3</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>1660.35</v>
+        <v>4905.68</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>752.78</v>
+        <v>3702.29</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>15142.09</v>
+        <v>63005.85</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Salaries &amp; Wages: Indirect /Purchase</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3916,47 +3916,47 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>courier, flags/badges, miscellaneous</t>
+          <t>purchasing</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>2138.76</v>
+        <v>5000</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1089.69</v>
+        <v>5000</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1123.01</v>
+        <v>5000</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>3789.07</v>
+        <v>5000</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>1320.49</v>
+        <v>4458</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>989.6799999999999</v>
+        <v>5000</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>1127.98</v>
+        <v>5000</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>1253.75</v>
+        <v>5000</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>508.94</v>
+        <v>5000</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>264.83</v>
+        <v>5000</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>316.45</v>
+        <v>4758</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>88.53</v>
+        <v>4958.33</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>14011.18</v>
+        <v>59174.33</v>
       </c>
     </row>
     <row r="36">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Utilities Expenses</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3977,52 +3977,52 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>stationery, printer ink, newspapers</t>
+          <t>ADDC electricity/water, Etisalat telephone and internet</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>783.13</v>
+        <v>4780.25</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>449.05</v>
+        <v>4568.37</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>373</v>
+        <v>4510.14</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>1618.98</v>
+        <v>4191.56</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>404.77</v>
+        <v>8334.92</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1228.67</v>
+        <v>4350.26</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>340.61</v>
+        <v>4242.75</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>481.01</v>
+        <v>4051.47</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>1156.65</v>
+        <v>4127.37</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>440.57</v>
+        <v>4358.95</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>237.4</v>
+        <v>4242.9</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>375.55</v>
+        <v>4322.62</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>7889.39</v>
+        <v>56081.56</v>
       </c>
     </row>
     <row r="37">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Claim Rejection</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4043,63 +4043,63 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>written-off rejected claims</t>
+          <t>Meta/WhatsApp API, Adobe, promotions</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>0</v>
+        <v>5820.11</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>0</v>
+        <v>2380.86</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>844.2</v>
+        <v>4382.51</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>0</v>
+        <v>4044.86</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0</v>
+        <v>4998.58</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>245</v>
+        <v>8392.940000000001</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>0</v>
+        <v>3713.11</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>0</v>
+        <v>5896.89</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>1005</v>
+        <v>2707.23</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>-32</v>
+        <v>1973.75</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>1235</v>
+        <v>8600.299999999999</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>105</v>
+        <v>2478.75</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>3402.2</v>
+        <v>55389.89</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): OHF</t>
+          <t>Salaries &amp; Wages: Indirect/Accounts</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4109,63 +4109,63 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>pantry and stationery issued from stock</t>
+          <t>accounts</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>1007.8</v>
+        <v>4645</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>0</v>
+        <v>3355</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0</v>
+        <v>3956</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0</v>
+        <v>4391</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>0</v>
+        <v>4938</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0</v>
+        <v>3975</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0</v>
+        <v>4090</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0</v>
+        <v>4016</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>0</v>
+        <v>4658</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>0</v>
+        <v>4656.25</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>1007.8</v>
+        <v>51180.25</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect it</t>
+          <t>Legal &amp; Professional Expenses: on-cost → OHF</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4175,63 +4175,63 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Overhead — IT</t>
+          <t>Overhead — back-office staff on-costs</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0</v>
+        <v>5581.24</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>0</v>
+        <v>1257.72</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0</v>
+        <v>1551.11</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>0</v>
+        <v>2404.58</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0</v>
+        <v>3524.51</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>0</v>
+        <v>8214.450000000001</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>0</v>
+        <v>2794.54</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0</v>
+        <v>4680.02</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0</v>
+        <v>3762.83</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0</v>
+        <v>2436.96</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>0</v>
+        <v>4293.9</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>0</v>
+        <v>3242.1</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>0</v>
+        <v>43743.96</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+          <t>Repair &amp; Maintenance Expenses</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4241,118 +4241,118 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Overhead — HR</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>general premises maintenance supplies and works</t>
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0</v>
+        <v>3948.75</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>0</v>
+        <v>701.2</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>0</v>
+        <v>1519</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>0</v>
+        <v>2904.65</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0</v>
+        <v>418.3</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>0</v>
+        <v>579.13</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0</v>
+        <v>3615.85</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0</v>
+        <v>4075.55</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0</v>
+        <v>4223.2</v>
       </c>
       <c r="P40" s="3" t="n">
-        <v>0</v>
+        <v>2824</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>0</v>
+        <v>704.67</v>
       </c>
       <c r="R40" s="3" t="n">
-        <v>0</v>
+        <v>29014.3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Depreciation: furniture, office equipment, computers, software</t>
+          <t>Travelling &amp; Transportation</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>OHDepreciation</t>
+          <t>OHF</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Overhead — facility / IT</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+          <t>taxis, parking, petrol, car wash</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>2524.8</v>
+        <v>1620.78</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>2524.8</v>
+        <v>2671.44</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>2524.8</v>
+        <v>1406.51</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>2524.8</v>
+        <v>2252.91</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>2524.8</v>
+        <v>2285.53</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>2524.8</v>
+        <v>1225.52</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>2524.8</v>
+        <v>5340.97</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>2524.8</v>
+        <v>1464.2</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>2524.8</v>
+        <v>1523</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>2524.8</v>
+        <v>3348</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>2524.8</v>
+        <v>2184.07</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>2524.8</v>
+        <v>2346.5</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>30297.6</v>
+        <v>27669.43</v>
       </c>
     </row>
     <row r="42">
@@ -4363,176 +4363,836 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>Fines</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Overhead — administration</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>1635</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>263</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>1278</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>1031</v>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="3" t="n">
+        <v>8435.120000000001</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>1503</v>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="3" t="n">
+        <v>2242.91</v>
+      </c>
+      <c r="Q42" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>17013.03</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Overhead — back office</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>1576.08</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>1074.12</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>748.9299999999999</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>1483.1</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>705.55</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>1314.1</v>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>1310.92</v>
+      </c>
+      <c r="M43" s="3" t="n">
+        <v>1821.61</v>
+      </c>
+      <c r="N43" s="3" t="n">
+        <v>1056.15</v>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>1638.4</v>
+      </c>
+      <c r="P43" s="3" t="n">
+        <v>1660.35</v>
+      </c>
+      <c r="Q43" s="3" t="n">
+        <v>752.78</v>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>15142.09</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Overhead — administration</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>courier, flags/badges, miscellaneous</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>2138.76</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>1089.69</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>1123.01</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>3789.07</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>1320.49</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>989.6799999999999</v>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>1127.98</v>
+      </c>
+      <c r="M44" s="3" t="n">
+        <v>1253.75</v>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>508.94</v>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>264.83</v>
+      </c>
+      <c r="P44" s="3" t="n">
+        <v>316.45</v>
+      </c>
+      <c r="Q44" s="3" t="n">
+        <v>88.53</v>
+      </c>
+      <c r="R44" s="3" t="n">
+        <v>14011.18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Insurance: on-cost → OHF</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Overhead — back-office staff on-costs</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>1055.81</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>881.28</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>1050.52</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>1516.22</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>1448.93</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>1579.89</v>
+      </c>
+      <c r="L45" s="3" t="n">
+        <v>1382.3</v>
+      </c>
+      <c r="M45" s="3" t="n">
+        <v>546.45</v>
+      </c>
+      <c r="N45" s="3" t="n">
+        <v>565.1799999999999</v>
+      </c>
+      <c r="O45" s="3" t="n">
+        <v>503.13</v>
+      </c>
+      <c r="P45" s="3" t="n">
+        <v>587.6900000000001</v>
+      </c>
+      <c r="Q45" s="3" t="n">
+        <v>540.89</v>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>11658.29</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Overhead — administration</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>stationery, printer ink, newspapers</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>783.13</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>449.05</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>373</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>1618.98</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>404.77</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>1228.67</v>
+      </c>
+      <c r="L46" s="3" t="n">
+        <v>340.61</v>
+      </c>
+      <c r="M46" s="3" t="n">
+        <v>481.01</v>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>1156.65</v>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>440.57</v>
+      </c>
+      <c r="P46" s="3" t="n">
+        <v>237.4</v>
+      </c>
+      <c r="Q46" s="3" t="n">
+        <v>375.55</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>7889.39</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Claim Rejection</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Overhead — patient administration</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>written-off rejected claims</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>844.2</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>245</v>
+      </c>
+      <c r="L47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="3" t="n">
+        <v>1005</v>
+      </c>
+      <c r="O47" s="3" t="n">
+        <v>-32</v>
+      </c>
+      <c r="P47" s="3" t="n">
+        <v>1235</v>
+      </c>
+      <c r="Q47" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="R47" s="3" t="n">
+        <v>3402.2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Stock movement</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cost of Goods Sold (M01): OHF</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Overhead — back office</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>pantry and stationery issued from stock</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>1007.8</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" s="3" t="n">
+        <v>1007.8</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Salary sheet</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Salaries &amp; Wages: Indirect it</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Overhead — IT</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Salary sheet</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Overhead — HR</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TB depreciation</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Depreciation: furniture, office equipment, computers, software</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Overhead — facility / IT</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="L51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="M51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="N51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="O51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="P51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="Q51" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="R51" s="3" t="n">
+        <v>30297.6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Monthly sheet</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>Third Party &amp; Professional Services</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>OHC</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Overhead — shared services</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>MySmyle Company EMR subscription, management consultancy and IT services (25,000/month) + Calibrate/Platform Technologies: services charged by a sister company = corporate/shared-services overhead</t>
         </is>
       </c>
-      <c r="F42" s="3" t="n">
+      <c r="F52" s="3" t="n">
         <v>8317</v>
       </c>
-      <c r="G42" s="3" t="n">
+      <c r="G52" s="3" t="n">
         <v>37300</v>
       </c>
-      <c r="H42" s="3" t="n">
+      <c r="H52" s="3" t="n">
         <v>62270</v>
       </c>
-      <c r="I42" s="3" t="n">
+      <c r="I52" s="3" t="n">
         <v>66480.95</v>
       </c>
-      <c r="J42" s="3" t="n">
+      <c r="J52" s="3" t="n">
         <v>2500</v>
       </c>
-      <c r="K42" s="3" t="n">
+      <c r="K52" s="3" t="n">
         <v>37375.73</v>
       </c>
-      <c r="L42" s="3" t="n">
+      <c r="L52" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="M42" s="3" t="n">
+      <c r="M52" s="3" t="n">
         <v>27500</v>
       </c>
-      <c r="N42" s="3" t="n">
+      <c r="N52" s="3" t="n">
         <v>28000</v>
       </c>
-      <c r="O42" s="3" t="n">
+      <c r="O52" s="3" t="n">
         <v>25500</v>
       </c>
-      <c r="P42" s="3" t="n">
+      <c r="P52" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="Q42" s="3" t="n">
+      <c r="Q52" s="3" t="n">
         <v>25104.5</v>
       </c>
-      <c r="R42" s="3" t="n">
+      <c r="R52" s="3" t="n">
         <v>370348.18</v>
       </c>
     </row>
-    <row r="43">
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="n"/>
-      <c r="L43" s="3" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="N43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
-      <c r="P43" s="3" t="n"/>
-      <c r="Q43" s="3" t="n"/>
-      <c r="R43" s="3" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-      <c r="B44" s="4" t="inlineStr">
+    <row r="53">
+      <c r="F53" s="3" t="n"/>
+      <c r="G53" s="3" t="n"/>
+      <c r="H53" s="3" t="n"/>
+      <c r="I53" s="3" t="n"/>
+      <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
+      <c r="L53" s="3" t="n"/>
+      <c r="M53" s="3" t="n"/>
+      <c r="N53" s="3" t="n"/>
+      <c r="O53" s="3" t="n"/>
+      <c r="P53" s="3" t="n"/>
+      <c r="Q53" s="3" t="n"/>
+      <c r="R53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr"/>
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>TOTAL mapped</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="5" t="n">
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="5" t="n">
         <v>511302.3</v>
       </c>
-      <c r="G44" s="5" t="n">
+      <c r="G54" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H44" s="5" t="n">
+      <c r="H54" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I44" s="5" t="n">
+      <c r="I54" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J44" s="5" t="n">
+      <c r="J54" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K44" s="5" t="n">
+      <c r="K54" s="5" t="n">
         <v>616494.08</v>
       </c>
-      <c r="L44" s="5" t="n">
+      <c r="L54" s="5" t="n">
         <v>480166.81</v>
       </c>
-      <c r="M44" s="5" t="n">
+      <c r="M54" s="5" t="n">
         <v>526990.09</v>
       </c>
-      <c r="N44" s="5" t="n">
+      <c r="N54" s="5" t="n">
         <v>509542.04</v>
       </c>
-      <c r="O44" s="5" t="n">
+      <c r="O54" s="5" t="n">
         <v>546725.96</v>
       </c>
-      <c r="P44" s="5" t="n">
+      <c r="P54" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q44" s="5" t="n">
+      <c r="Q54" s="5" t="n">
         <v>623033.72</v>
       </c>
-      <c r="R44" s="5" t="n">
+      <c r="R54" s="5" t="n">
         <v>6453401.91</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr"/>
-      <c r="B45" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Ledger (locked)</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="5" t="n">
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="5" t="n">
         <v>511302.3</v>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G55" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H55" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I55" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J45" s="5" t="n">
+      <c r="J55" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K45" s="5" t="n">
+      <c r="K55" s="5" t="n">
         <v>616494.09</v>
       </c>
-      <c r="L45" s="5" t="n">
+      <c r="L55" s="5" t="n">
         <v>480166.82</v>
       </c>
-      <c r="M45" s="5" t="n">
+      <c r="M55" s="5" t="n">
         <v>526990.1</v>
       </c>
-      <c r="N45" s="5" t="n">
+      <c r="N55" s="5" t="n">
         <v>509542.05</v>
       </c>
-      <c r="O45" s="5" t="n">
+      <c r="O55" s="5" t="n">
         <v>546725.98</v>
       </c>
-      <c r="P45" s="5" t="n">
+      <c r="P55" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q45" s="5" t="n">
+      <c r="Q55" s="5" t="n">
         <v>623033.73</v>
       </c>
-      <c r="R45" s="5" t="n">
+      <c r="R55" s="5" t="n">
         <v>6453401.98</v>
       </c>
     </row>
@@ -4570,7 +5230,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q2. Staff Qualification And Education (889,431.99) is mapped to OHF (HR administration and IT). If part of it is staff on-costs of the dentists and nurses (visas, licences, benefits), that part belongs with SWDoc/SWNurs and the overhead ratio falls (to roughly 34% if all of it were on-costs).</t>
+          <t>Q2. Staff on-costs (Staff Qualification And Education 889,431.99 in full; Insurance 50,409.29 in full; clinician licences 34,349.57 and visas / labour 145,165.32 out of Legal &amp; Professional) are split every month by the salary share of dentists / nurses / CSSD + technicians / back office, employees only (ruling 13 Oct 2026). The rest of Legal &amp; Professional (facility licences, accreditation, trade licence, civil defence, tenancy) stays OHF.</t>
         </is>
       </c>
     </row>
@@ -4598,7 +5258,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Overhead ratio by month: 01 36.3%, 02 31.1%, 03 38.0%, 04 44.7%, 05 39.8%, 06 58.1%, 07 52.1%, 08 50.6%, 09 50.3%, 10 46.5%, 11 46.1%, 12 47.5%; FY2025 45.2% (DOH band 20% to under 50%)</t>
+          <t>Overhead ratio by month: 01 25.7%, 02 26.7%, 03 30.0%, 04 36.9%, 05 28.0%, 06 35.2%, 07 34.8%, 08 35.1%, 09 36.9%, 10 32.5%, 11 36.9%, 12 29.7%; FY2025 32.3% (DOH band 20% to under 50%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruling: staff on-costs by the nature of each cost (salary, headcount, licensed headcount); refill ledger map; re-run January
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -553,40 +553,40 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>31532.24</v>
+        <v>36730.81</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>28267.94</v>
+        <v>29995.57</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30636.78</v>
+        <v>32617.62</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>31474.11</v>
+        <v>33952.2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>37720.38</v>
+        <v>40465.14</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>53560.11</v>
+        <v>59199.4</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>41977.45</v>
+        <v>43481.96</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>45741.97</v>
+        <v>47559.49</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>29312.81</v>
+        <v>30923.73</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>40078.65</v>
+        <v>41560.81</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>36879.04</v>
+        <v>38852.45</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>44482.71</v>
+        <v>46401.93</v>
       </c>
       <c r="O2" s="3">
         <f>SUM(C2:N2)</f>
@@ -605,40 +605,40 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>215914.15</v>
+        <v>202921.41</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>246035.58</v>
+        <v>240908</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>247548.14</v>
+        <v>241587.59</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>169173.03</v>
+        <v>163755.24</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>197696.32</v>
+        <v>191193.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>244323.08</v>
+        <v>232448.65</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>168978.6</v>
+        <v>165564.06</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>159401.46</v>
+        <v>155839.06</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>175914.16</v>
+        <v>172177.1</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>223880.42</v>
+        <v>220195.09</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>163006.68</v>
+        <v>158753.06</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>251434.38</v>
+        <v>246757.2</v>
       </c>
       <c r="O3" s="3">
         <f>SUM(C3:N3)</f>
@@ -657,40 +657,40 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>17776.15</v>
+        <v>20665.2</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13735.31</v>
+        <v>14984.34</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>15109.63</v>
+        <v>16447.64</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>11787.67</v>
+        <v>13193.46</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>15640.89</v>
+        <v>17094.45</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>12864.73</v>
+        <v>14851.9</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>16822.55</v>
+        <v>18203.87</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>22996.09</v>
+        <v>24282.36</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>20817.73</v>
+        <v>22115.57</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>16981.43</v>
+        <v>18079.73</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>19135.63</v>
+        <v>20429.83</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>30723.69</v>
+        <v>32189.55</v>
       </c>
       <c r="O4" s="3">
         <f>SUM(C4:N4)</f>
@@ -1177,40 +1177,40 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>120691.66</v>
+        <v>125596.78</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>102214.03</v>
+        <v>104364.95</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>117405.5</v>
+        <v>120047.2</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>122171.09</v>
+        <v>123705</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>131752.15</v>
+        <v>134056.35</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>176906.62</v>
+        <v>181154.59</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>139524.14</v>
+        <v>140052.85</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>155046.62</v>
+        <v>155505.23</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>157279.78</v>
+        <v>158108.08</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>149470.76</v>
+        <v>150575.63</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>154884.87</v>
+        <v>155870.88</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>157673.67</v>
+        <v>158965.77</v>
       </c>
       <c r="O14" s="3">
         <f>SUM(C14:N14)</f>
@@ -1613,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education: on-cost → SWNurs</t>
+          <t>Staff Qualification And Education: benefits, bonus, end-of-service, training → SWNurs</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly salary key (Nurse/licensed, Nurse/No License); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses: on-cost → SWNurs</t>
+          <t>Legal &amp; Professional Expenses: visas, work permits, labour cards → SWNurs</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1936,47 +1936,47 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly headcount key (Nurse/licensed, Nurse/No License); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>3069.24</v>
+        <v>5345.12</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>713.37</v>
+        <v>1313.36</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>759.46</v>
+        <v>1426.73</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1047.57</v>
+        <v>1915.54</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>1661.75</v>
+        <v>2680.45</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>3957.36</v>
+        <v>6302.34</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1185.41</v>
+        <v>1622.03</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>2209.4</v>
+        <v>2759.87</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>1216.68</v>
+        <v>1932.71</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1016.65</v>
+        <v>1611.14</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>1784.8</v>
+        <v>2509.13</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>1329.74</v>
+        <v>2103.55</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>19951.43</v>
+        <v>31521.97</v>
       </c>
     </row>
     <row r="6">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Insurance: on-cost → SWNurs</t>
+          <t>Legal &amp; Professional Expenses: clinician licences (DOH, Dataflow, CME) → SWNurs</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2002,124 +2002,124 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Nurse/licensed, Nurse/No License (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly licensed key (Nurse/licensed); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>580.61</v>
+        <v>2252.9</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>499.86</v>
+        <v>489.47</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>514.36</v>
+        <v>633</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>660.5599999999999</v>
+        <v>777.02</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>683.15</v>
+        <v>1046.53</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>761.12</v>
+        <v>2556.48</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>586.36</v>
+        <v>662.0700000000001</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>257.97</v>
+        <v>1126.52</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>182.75</v>
+        <v>718.65</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>209.89</v>
+        <v>686.22</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>244.28</v>
+        <v>1068.69</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>221.85</v>
+        <v>933.28</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>5402.76</v>
+        <v>12950.83</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Direct Dr</t>
+          <t>Insurance: staff medical insurance → SWNurs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SWDoc</t>
+          <t>SWNurs</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — dental surgeries (nurses' on-costs)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>dentists, oral surgeon, orthodontist (Salary sheet 'Direct Dr')</t>
+          <t>staff on-cost; monthly headcount key (Nurse/licensed, Nurse/No License); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>171870</v>
+        <v>1250.4</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>225878.31</v>
+        <v>1138.03</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>206907</v>
+        <v>1194.93</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>136987</v>
+        <v>1493.66</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>152254</v>
+        <v>1362.68</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>132942</v>
+        <v>1498.95</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>107479</v>
+        <v>992.1799999999999</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>102568</v>
+        <v>398.5</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>122528</v>
+        <v>358.99</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>162693</v>
+        <v>411.34</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>129357.35</v>
+        <v>424.67</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>166275.01</v>
+        <v>433.98</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>1817738.67</v>
+        <v>10958.31</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education: on-cost → SWDoc</t>
+          <t>Salaries &amp; Wages: Direct Dr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2129,52 +2129,52 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries (dentists' on-costs)</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
+          <t>dentists, oral surgeon, orthodontist (Salary sheet 'Direct Dr')</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>19052.18</v>
+        <v>171870</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>9597.66</v>
+        <v>225878.31</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>30348.52</v>
+        <v>206907</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>23004.85</v>
+        <v>136987</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>33152.46</v>
+        <v>152254</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>89856.97</v>
+        <v>132942</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>54367.39</v>
+        <v>107479</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>48235.17</v>
+        <v>102568</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>44987.84</v>
+        <v>122528</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>54335.9</v>
+        <v>162693</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>24680.75</v>
+        <v>129357.35</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>76389.19</v>
+        <v>166275.01</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>508008.88</v>
+        <v>1817738.67</v>
       </c>
     </row>
     <row r="9">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses: on-cost → SWDoc</t>
+          <t>Staff Qualification And Education: benefits, bonus, end-of-service, training → SWDoc</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2200,47 +2200,47 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly salary key (Direct Dr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>21016.31</v>
+        <v>19052.18</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>6208.98</v>
+        <v>9597.66</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>6136.53</v>
+        <v>30348.52</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>5630.7</v>
+        <v>23004.85</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>8709.41</v>
+        <v>33152.46</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>18052.14</v>
+        <v>89856.97</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>4771.84</v>
+        <v>54367.39</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>7699.3</v>
+        <v>48235.17</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>7301.61</v>
+        <v>44987.84</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>5679.04</v>
+        <v>54335.9</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>7888.87</v>
+        <v>24680.75</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>7516.23</v>
+        <v>76389.19</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>106610.96</v>
+        <v>508008.88</v>
       </c>
     </row>
     <row r="10">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Insurance: on-cost → SWDoc</t>
+          <t>Legal &amp; Professional Expenses: visas, work permits, labour cards → SWDoc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2266,190 +2266,190 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Direct Dr (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly headcount key (Direct Dr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>3975.66</v>
+        <v>6681.41</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>4350.63</v>
+        <v>2298.39</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4156.09</v>
+        <v>1783.42</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>3550.48</v>
+        <v>1532.43</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>3580.45</v>
+        <v>2680.45</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>3471.97</v>
+        <v>5041.87</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>2360.37</v>
+        <v>1622.03</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>898.99</v>
+        <v>2759.87</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>1096.71</v>
+        <v>2415.89</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>1172.48</v>
+        <v>1611.14</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>1079.71</v>
+        <v>2509.13</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>1253.95</v>
+        <v>2103.55</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>30947.49</v>
+        <v>33039.58</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Cssd</t>
+          <t>Legal &amp; Professional Expenses: clinician licences (DOH, Dataflow, CME) → SWDoc</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SWAllied</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Direct — CSSD (cost centre 07)</t>
+          <t>Direct — dental surgeries (dentists' on-costs)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sterilisation technicians</t>
+          <t>staff on-cost; monthly licensed key (Direct Dr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>7000</v>
+        <v>3754.82</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>7000</v>
+        <v>1142.09</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>7000</v>
+        <v>1054.99</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>6500</v>
+        <v>1036.03</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>7000</v>
+        <v>1744.21</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>7000</v>
+        <v>3408.65</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>7000</v>
+        <v>1103.46</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>7000</v>
+        <v>1877.52</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>7500</v>
+        <v>1796.64</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>7500</v>
+        <v>1143.71</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>7500</v>
+        <v>1781.16</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>8000</v>
+        <v>1555.47</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>86000</v>
+        <v>21398.75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/LAB</t>
+          <t>Insurance: staff medical insurance → SWDoc</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SWAllied</t>
+          <t>SWDoc</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Direct — prostheses (cost centre 09, in-house CAD/CAM)</t>
+          <t>Direct — dental surgeries (dentists' on-costs)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>dental technicians making prostheses; routed to the Prosthesis bucket on prosthesis claims (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly headcount key (Direct Dr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>7150</v>
+        <v>1563</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>5610</v>
+        <v>1991.55</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>5629</v>
+        <v>1493.66</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>3045</v>
+        <v>1194.93</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>5045.69</v>
+        <v>1362.68</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0</v>
+        <v>1199.16</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>3700</v>
+        <v>992.1799999999999</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>7797</v>
+        <v>398.5</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>7000</v>
+        <v>448.73</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>4840.34</v>
+        <v>411.34</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>7685.48</v>
+        <v>424.67</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>12317.75</v>
+        <v>433.98</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>69820.25999999999</v>
+        <v>11914.38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education: on-cost → SWAllied</t>
+          <t>Salaries &amp; Wages: Cssd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2459,63 +2459,63 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
+          <t>Direct — CSSD (cost centre 07)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
+          <t>sterilisation technicians</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1568.56</v>
+        <v>7000</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>535.8</v>
+        <v>7000</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1852.39</v>
+        <v>7000</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1602.94</v>
+        <v>6500</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>2622.88</v>
+        <v>7000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>4731.38</v>
+        <v>7000</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>5412.51</v>
+        <v>7000</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>6958.66</v>
+        <v>7000</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>5323.87</v>
+        <v>7500</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>4121.4</v>
+        <v>7500</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>2897.31</v>
+        <v>7500</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>9334.27</v>
+        <v>8000</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>46961.97</v>
+        <v>86000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses: on-cost → SWAllied</t>
+          <t>Salaries &amp; Wages: Indirect/LAB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2525,52 +2525,52 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
+          <t>Direct — prostheses (cost centre 09, in-house CAD/CAM)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
+          <t>dental technicians making prostheses; routed to the Prosthesis bucket on prosthesis claims (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1730.27</v>
+        <v>7150</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>346.63</v>
+        <v>5610</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>374.56</v>
+        <v>5629</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>392.34</v>
+        <v>3045</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>689.05</v>
+        <v>5045.69</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>950.53</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>475.06</v>
+        <v>3700</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>1110.74</v>
+        <v>7797</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>864.0700000000001</v>
+        <v>7000</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>430.76</v>
+        <v>4840.34</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>926.09</v>
+        <v>7685.48</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>918.4400000000001</v>
+        <v>12317.75</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>9208.540000000001</v>
+        <v>69820.25999999999</v>
       </c>
     </row>
     <row r="15">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Insurance: on-cost → SWAllied</t>
+          <t>Staff Qualification And Education: benefits, bonus, end-of-service, training → SWAllied</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2596,179 +2596,179 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Cssd, Indirect/LAB (ruling 13 Oct 2026)</t>
+          <t>staff on-cost; monthly salary key (Cssd, Indirect/LAB); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>327.32</v>
+        <v>1568.56</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>242.88</v>
+        <v>535.8</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>253.68</v>
+        <v>1852.39</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>247.39</v>
+        <v>1602.94</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>283.27</v>
+        <v>2622.88</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>182.82</v>
+        <v>4731.38</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>234.98</v>
+        <v>5412.51</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>129.69</v>
+        <v>6958.66</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>129.79</v>
+        <v>5323.87</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>88.93000000000001</v>
+        <v>4121.4</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>126.75</v>
+        <v>2897.31</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>153.23</v>
+        <v>9334.27</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>2400.73</v>
+        <v>46961.97</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Pharmacy</t>
+          <t>Legal &amp; Professional Expenses: visas, work permits, labour cards → SWAllied</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pharmacy</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
+          <t>staff on-cost; monthly headcount key (Cssd, Indirect/LAB); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1252</v>
+        <v>4008.84</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0</v>
+        <v>985.02</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0</v>
+        <v>1070.05</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0</v>
+        <v>1149.32</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0</v>
+        <v>1608.27</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0</v>
+        <v>2520.94</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0</v>
+        <v>1297.62</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>2207.9</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0</v>
+        <v>1932.71</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0</v>
+        <v>1288.92</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0</v>
+        <v>2007.3</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0</v>
+        <v>2103.55</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>1252</v>
+        <v>22180.44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Internal LAB</t>
+          <t>Insurance: staff medical insurance → SWAllied</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>SWAllied</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — CSSD / prostheses (technicians' on-costs)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
+          <t>staff on-cost; monthly headcount key (Cssd, Indirect/LAB); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0</v>
+        <v>937.8</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>18259.88</v>
+        <v>853.52</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>21431.24</v>
+        <v>896.2</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>21431.24</v>
+        <v>896.2</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>7316.68</v>
+        <v>817.61</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>13158.04</v>
+        <v>599.58</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>13819.96</v>
+        <v>793.74</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>20017.81</v>
+        <v>318.8</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>16858.99</v>
+        <v>358.99</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>18917.63</v>
+        <v>329.07</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>15006.23</v>
+        <v>339.74</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>15194.75</v>
+        <v>433.98</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>181412.45</v>
+        <v>7575.23</v>
       </c>
     </row>
     <row r="18">
@@ -2779,26 +2779,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Prostheses</t>
+          <t>Cost of Goods Sold (M01): Pharmacy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Prostheses</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
+          <t>local anaesthetic cartridges, nitrous oxide and oxygen</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>68204.94</v>
+        <v>1252</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>0</v>
@@ -2834,18 +2834,18 @@
         <v>0</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>68204.94</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>External Lab</t>
+          <t>Cost of Goods Sold: Internal LAB</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2860,58 +2860,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
+          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1870</v>
+        <v>0</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>200</v>
+        <v>18259.88</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>16430</v>
+        <v>21431.24</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>4288</v>
+        <v>21431.24</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>7425</v>
+        <v>7316.68</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0</v>
+        <v>13158.04</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>5270</v>
+        <v>13819.96</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>6381</v>
+        <v>20017.81</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>1150</v>
+        <v>16858.99</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>950</v>
+        <v>18917.63</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>10595</v>
+        <v>15006.23</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>12186.25</v>
+        <v>15194.75</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>66745.25</v>
+        <v>181412.45</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: External LAB</t>
+          <t>Cost of Goods Sold (M01): Prostheses</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2921,118 +2921,118 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>prostheses bought from external laboratories, booked in cost of goods sold</t>
+          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>68204.94</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>7285</v>
+        <v>0</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1735</v>
+        <v>0</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>7425</v>
+        <v>0</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>4810</v>
+        <v>0</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>5254</v>
+        <v>0</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>10987.5</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>12557.75</v>
+        <v>0</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>52354.25</v>
+        <v>68204.94</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -( Dr</t>
+          <t>External Lab</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>clinical consumables issued to the dental surgeries</t>
+          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0</v>
+        <v>1870</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>67171.58</v>
+        <v>200</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>70803.81</v>
+        <v>16430</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>70803.81</v>
+        <v>4288</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>63371.43</v>
+        <v>7425</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>61129.96</v>
+        <v>0</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>46785.8</v>
+        <v>5270</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>67034.7</v>
+        <v>6381</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>62943.56</v>
+        <v>1150</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>51591.7</v>
+        <v>950</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>39376.22</v>
+        <v>10595</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>50594.58</v>
+        <v>12186.25</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>651607.15</v>
+        <v>66745.25</v>
       </c>
     </row>
     <row r="22">
@@ -3043,73 +3043,73 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
+          <t>Cost of Goods Sold: External LAB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Prostheses</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Direct — CSSD</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>sterilisation and vital-signs consumables</t>
+          <t>prostheses bought from external laboratories, booked in cost of goods sold</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>3617.35</v>
+        <v>200</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>4867.36</v>
+        <v>7285</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>4867.36</v>
+        <v>1735</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>4137.43</v>
+        <v>7425</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>4094.41</v>
+        <v>0</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>4096.91</v>
+        <v>4810</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>4535.04</v>
+        <v>5254</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>3033.61</v>
+        <v>1150</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>3973.98</v>
+        <v>950</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>5793.45</v>
+        <v>10987.5</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>9800.040000000001</v>
+        <v>12557.75</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>52816.94</v>
+        <v>52354.25</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): MS</t>
+          <t>Cost of Goods Sold: Consumables -( Dr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3119,316 +3119,316 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / CSSD</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
+          <t>clinical consumables issued to the dental surgeries</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>31662.75</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0</v>
+        <v>67171.58</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0</v>
+        <v>70803.81</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>70803.81</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0</v>
+        <v>63371.43</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0</v>
+        <v>61129.96</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0</v>
+        <v>46785.8</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0</v>
+        <v>67034.7</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0</v>
+        <v>62943.56</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>0</v>
+        <v>51591.7</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>0</v>
+        <v>39376.22</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>0</v>
+        <v>50594.58</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>31662.75</v>
+        <v>651607.15</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Equipment Maintenanace</t>
+          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — CSSD</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>maintenance of dental chairs and clinical equipment</t>
+          <t>sterilisation and vital-signs consumables</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>2258.57</v>
+        <v>3617.35</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0</v>
+        <v>4867.36</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>830</v>
+        <v>4867.36</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0</v>
+        <v>4137.43</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0</v>
+        <v>4094.41</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0</v>
+        <v>4096.91</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0</v>
+        <v>4535.04</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0</v>
+        <v>3033.61</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>1350</v>
+        <v>3973.98</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>0</v>
+        <v>5793.45</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>200</v>
+        <v>9800.040000000001</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>5638.57</v>
+        <v>52816.94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Depreciation: Machinery &amp; Equipment</t>
+          <t>Cost of Goods Sold (M01): MS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / imaging</t>
+          <t>Direct — dental surgeries / CSSD</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
+          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>10556.61</v>
+        <v>31662.75</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>10556.61</v>
+        <v>0</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>126679.32</v>
+        <v>31662.75</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Management</t>
+          <t>Equipment Maintenanace</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Overhead — management</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>clinic management</t>
+          <t>maintenance of dental chairs and clinical equipment</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>20000</v>
+        <v>1000</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>20000</v>
+        <v>2258.57</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>28000</v>
+        <v>830</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>28000</v>
+        <v>1350</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>28000</v>
+        <v>200</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>310000</v>
+        <v>5638.57</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>TB depreciation</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Staff Qualification And Education: on-cost → OHF</t>
+          <t>Depreciation: Machinery &amp; Equipment</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OHF</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Overhead — back-office staff on-costs</t>
+          <t>Direct — dental surgeries / imaging</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HR administration: visas, work permits, staff benefits, final settlements, training, licences, information-management (IT) charges; staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
+          <t>dental chairs, imaging units, autoclaves (2025 charge 126,679.42)</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5059.63</v>
+        <v>10556.61</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1944.15</v>
+        <v>10556.61</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>7671.07</v>
+        <v>10556.61</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>9824.17</v>
+        <v>10556.61</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>13416.1</v>
+        <v>10556.61</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>40888.57</v>
+        <v>10556.61</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>31839.21</v>
+        <v>10556.61</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>29319.77</v>
+        <v>10556.61</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>23184.18</v>
+        <v>10556.61</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>23316.35</v>
+        <v>10556.61</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>13433.69</v>
+        <v>10556.61</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>32950.18</v>
+        <v>10556.61</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>232847.07</v>
+        <v>126679.32</v>
       </c>
     </row>
     <row r="28">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/RAP</t>
+          <t>Salaries &amp; Wages: Indirect /Management</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3449,63 +3449,63 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Overhead — reception / patient administration</t>
+          <t>Overhead — management</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>reception and patient-administration staff</t>
+          <t>clinic management</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>11598</v>
+        <v>20000</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>12400</v>
+        <v>20000</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>12232</v>
+        <v>20000</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>10000</v>
+        <v>28000</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>14200</v>
+        <v>27000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>13700</v>
+        <v>27000</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>13669</v>
+        <v>28000</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>14500</v>
+        <v>28000</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>15000</v>
+        <v>28000</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>21550</v>
+        <v>28000</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>21759</v>
+        <v>28000</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>22125</v>
+        <v>28000</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>182733</v>
+        <v>310000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: External</t>
+          <t>Staff Qualification And Education: benefits, bonus, end-of-service, training → OHF</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3515,52 +3515,52 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back-office staff on-costs</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
+          <t>staff on-cost; monthly salary key (Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>7600</v>
+        <v>5059.63</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>12690</v>
+        <v>1944.15</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>11520</v>
+        <v>7671.07</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>9505</v>
+        <v>9824.17</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>7800</v>
+        <v>13416.1</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>9070</v>
+        <v>40888.57</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>9700</v>
+        <v>31839.21</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>11596</v>
+        <v>29319.77</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>16600</v>
+        <v>23184.18</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>15600</v>
+        <v>23316.35</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>15600</v>
+        <v>13433.69</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>15600</v>
+        <v>32950.18</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>142881</v>
+        <v>232847.07</v>
       </c>
     </row>
     <row r="30">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /INS</t>
+          <t>Salaries &amp; Wages: Indirect/RAP</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3581,63 +3581,63 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — reception / patient administration</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>insurance claims staff</t>
+          <t>reception and patient-administration staff</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>4400</v>
+        <v>11598</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>5000</v>
+        <v>12400</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>10567</v>
+        <v>12232</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>11500</v>
+        <v>10000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>12000</v>
+        <v>14200</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>10403</v>
+        <v>13700</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>11336</v>
+        <v>13669</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>10871</v>
+        <v>14500</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>11054</v>
+        <v>15000</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>11248</v>
+        <v>21550</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>11234</v>
+        <v>21759</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>11982.5</v>
+        <v>22125</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>121595.5</v>
+        <v>182733</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Clinic Rent</t>
+          <t>Salaries &amp; Wages: External</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3647,63 +3647,63 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
+          <t>external accountant, drivers, cleaners and other outsourced support staff</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>7083.33</v>
+        <v>7600</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>7083.33</v>
+        <v>12690</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>7083.33</v>
+        <v>11520</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>7083.33</v>
+        <v>9505</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>7083.33</v>
+        <v>7800</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>7083.33</v>
+        <v>9070</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>7083.33</v>
+        <v>9700</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>7083.33</v>
+        <v>11596</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>7083.33</v>
+        <v>16600</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>7083.33</v>
+        <v>15600</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>7083.33</v>
+        <v>15600</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>7083.33</v>
+        <v>15600</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>84999.96000000001</v>
+        <v>142881</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dues &amp; Subscriptions</t>
+          <t>Salaries &amp; Wages: Indirect /INS</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3713,52 +3713,52 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Overhead — IT / administration</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>software subscriptions, memberships</t>
+          <t>insurance claims staff</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>5585</v>
+        <v>4400</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>9203.280000000001</v>
+        <v>5000</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>8414.280000000001</v>
+        <v>10567</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>6503.7</v>
+        <v>12000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>10028.04</v>
+        <v>10403</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>99.54000000000001</v>
+        <v>11336</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>1842.43</v>
+        <v>10871</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>15774.05</v>
+        <v>11054</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>6523.81</v>
+        <v>11248</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>8884.18</v>
+        <v>11234</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>5667.86</v>
+        <v>11982.5</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>80526.17</v>
+        <v>121595.5</v>
       </c>
     </row>
     <row r="33">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses: non-on-cost part</t>
+          <t>Clinic Rent</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3779,52 +3779,52 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees (facility licences, accreditation, trade licence)</t>
+          <t>lease of the clinic premises (unit 1302, 85,000/year), allocated to the Dental bucket by floor space</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>12952.11</v>
+        <v>7083.33</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>3517.49</v>
+        <v>7083.33</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>3639.16</v>
+        <v>7083.33</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>3908.76</v>
+        <v>7083.33</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>6016.58</v>
+        <v>7083.33</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>12860.28</v>
+        <v>7083.33</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>3806.31</v>
+        <v>7083.33</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>6476.44</v>
+        <v>7083.33</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>5422.73</v>
+        <v>7083.33</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>3945.16</v>
+        <v>7083.33</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>6144.02</v>
+        <v>7083.33</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>5365.53</v>
+        <v>7083.33</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>74054.57000000001</v>
+        <v>84999.96000000001</v>
       </c>
     </row>
     <row r="34">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Finance Charges</t>
+          <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3845,63 +3845,63 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — IT / administration</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>bank and card charges</t>
+          <t>software subscriptions, memberships</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>6820.88</v>
+        <v>5585</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>6684.05</v>
+        <v>9203.280000000001</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>9269.73</v>
+        <v>8414.280000000001</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>5865.9</v>
+        <v>2000</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>5876.86</v>
+        <v>6503.7</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>4410.88</v>
+        <v>10028.04</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>3220.43</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>4136.27</v>
+        <v>1842.43</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>4080.58</v>
+        <v>15774.05</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>4032.3</v>
+        <v>6523.81</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>4905.68</v>
+        <v>8884.18</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>3702.29</v>
+        <v>5667.86</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>63005.85</v>
+        <v>80526.17</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect /Purchase</t>
+          <t>Legal &amp; Professional Expenses: non-on-cost part</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3916,47 +3916,47 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>purchasing</t>
+          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees (facility licences, accreditation, trade licence, civil defence, tenancy)</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>5000</v>
+        <v>12952.11</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>5000</v>
+        <v>3517.48</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>5000</v>
+        <v>3639.17</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>5000</v>
+        <v>3908.76</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>4458</v>
+        <v>6016.57</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>5000</v>
+        <v>12860.28</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>5000</v>
+        <v>3806.31</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>5000</v>
+        <v>6476.44</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>5000</v>
+        <v>5422.73</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>5000</v>
+        <v>3945.15</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>4758</v>
+        <v>6144.02</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>4958.33</v>
+        <v>5365.53</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>59174.33</v>
+        <v>74054.55</v>
       </c>
     </row>
     <row r="36">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Utilities Expenses</t>
+          <t>Finance Charges</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3977,63 +3977,63 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ADDC electricity/water, Etisalat telephone and internet</t>
+          <t>bank and card charges</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>4780.25</v>
+        <v>6820.88</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>4568.37</v>
+        <v>6684.05</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>4510.14</v>
+        <v>9269.73</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>4191.56</v>
+        <v>5865.9</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>8334.92</v>
+        <v>5876.86</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>4350.26</v>
+        <v>4410.88</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>4242.75</v>
+        <v>3220.43</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>4051.47</v>
+        <v>4136.27</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>4127.37</v>
+        <v>4080.58</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>4358.95</v>
+        <v>4032.3</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>4242.9</v>
+        <v>4905.68</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>4322.62</v>
+        <v>3702.29</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>56081.56</v>
+        <v>63005.85</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Salaries &amp; Wages: Indirect /Purchase</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4048,58 +4048,58 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Meta/WhatsApp API, Adobe, promotions</t>
+          <t>purchasing</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>5820.11</v>
+        <v>5000</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>2380.86</v>
+        <v>5000</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>4382.51</v>
+        <v>5000</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>4044.86</v>
+        <v>5000</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>4998.58</v>
+        <v>4458</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>8392.940000000001</v>
+        <v>5000</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>3713.11</v>
+        <v>5000</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>5896.89</v>
+        <v>5000</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>2707.23</v>
+        <v>5000</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>1973.75</v>
+        <v>5000</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>8600.299999999999</v>
+        <v>4758</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>2478.75</v>
+        <v>4958.33</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>55389.89</v>
+        <v>59174.33</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/Accounts</t>
+          <t>Legal &amp; Professional Expenses: visas, work permits, labour cards → OHF</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4109,52 +4109,52 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back-office staff on-costs</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>accounts</t>
+          <t>staff on-cost; monthly headcount key (Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>4645</v>
+        <v>9353.969999999999</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>3355</v>
+        <v>2298.38</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>4500</v>
+        <v>2853.46</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>4000</v>
+        <v>3064.85</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>3956</v>
+        <v>4824.82</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>4391</v>
+        <v>11344.2</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>4938</v>
+        <v>2919.64</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>3975</v>
+        <v>4967.78</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>4090</v>
+        <v>4348.59</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>4016</v>
+        <v>3222.29</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>4658</v>
+        <v>5018.25</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>4656.25</v>
+        <v>4207.11</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>51180.25</v>
+        <v>58423.34</v>
       </c>
     </row>
     <row r="39">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Expenses: on-cost → OHF</t>
+          <t>Utilities Expenses</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4175,52 +4175,52 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Overhead — back-office staff on-costs</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DOH facility/clinician licences, immigration and visas, trade licence, civil defence, ADHICS/Tasneef, typing/PRO fees; staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
+          <t>ADDC electricity/water, Etisalat telephone and internet</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>5581.24</v>
+        <v>4780.25</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>1257.72</v>
+        <v>4568.37</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>1551.11</v>
+        <v>4510.14</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>2404.58</v>
+        <v>4191.56</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>3524.51</v>
+        <v>8334.92</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>8214.450000000001</v>
+        <v>4350.26</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>2794.54</v>
+        <v>4242.75</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>4680.02</v>
+        <v>4051.47</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>3762.83</v>
+        <v>4127.37</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>2436.96</v>
+        <v>4358.95</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>4293.9</v>
+        <v>4242.9</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>3242.1</v>
+        <v>4322.62</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>43743.96</v>
+        <v>56081.56</v>
       </c>
     </row>
     <row r="40">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Repair &amp; Maintenance Expenses</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4241,63 +4241,63 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Overhead — facility</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>general premises maintenance supplies and works</t>
+          <t>Meta/WhatsApp API, Adobe, promotions</t>
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>3948.75</v>
+        <v>5820.11</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>701.2</v>
+        <v>2380.86</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1519</v>
+        <v>4382.51</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>2904.65</v>
+        <v>4044.86</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>418.3</v>
+        <v>4998.58</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>3500</v>
+        <v>8392.940000000001</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>579.13</v>
+        <v>3713.11</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>3615.85</v>
+        <v>5896.89</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>4075.55</v>
+        <v>2707.23</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>4223.2</v>
+        <v>1973.75</v>
       </c>
       <c r="P40" s="3" t="n">
-        <v>2824</v>
+        <v>8600.299999999999</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>704.67</v>
+        <v>2478.75</v>
       </c>
       <c r="R40" s="3" t="n">
-        <v>29014.3</v>
+        <v>55389.89</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Travelling &amp; Transportation</t>
+          <t>Salaries &amp; Wages: Indirect/Accounts</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4312,47 +4312,47 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>taxis, parking, petrol, car wash</t>
+          <t>accounts</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>1620.78</v>
+        <v>4645</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>2671.44</v>
+        <v>3355</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>1406.51</v>
+        <v>4500</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>2252.91</v>
+        <v>4000</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>2285.53</v>
+        <v>3956</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1225.52</v>
+        <v>4391</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>5340.97</v>
+        <v>4938</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>1464.2</v>
+        <v>3975</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>1523</v>
+        <v>4090</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>3348</v>
+        <v>4016</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>2184.07</v>
+        <v>4658</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>2346.5</v>
+        <v>4656.25</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>27669.43</v>
+        <v>51180.25</v>
       </c>
     </row>
     <row r="42">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Fines</t>
+          <t>Repair &amp; Maintenance Expenses</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4373,52 +4373,52 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — facility</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+          <t>general premises maintenance supplies and works</t>
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>1635</v>
+        <v>3948.75</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>263</v>
+        <v>701.2</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>0</v>
+        <v>1519</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1278</v>
+        <v>2904.65</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0</v>
+        <v>418.3</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1031</v>
+        <v>3500</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>0</v>
+        <v>579.13</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>8435.120000000001</v>
+        <v>3615.85</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>1503</v>
+        <v>4075.55</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0</v>
+        <v>4223.2</v>
       </c>
       <c r="P42" s="3" t="n">
-        <v>2242.91</v>
+        <v>2824</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>625</v>
+        <v>704.67</v>
       </c>
       <c r="R42" s="3" t="n">
-        <v>17013.03</v>
+        <v>29014.3</v>
       </c>
     </row>
     <row r="43">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Pantry</t>
+          <t>Travelling &amp; Transportation</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4439,52 +4439,52 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+          <t>taxis, parking, petrol, car wash</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1576.08</v>
+        <v>1620.78</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>1074.12</v>
+        <v>2671.44</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>748.9299999999999</v>
+        <v>1406.51</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>1483.1</v>
+        <v>2252.91</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>705.55</v>
+        <v>2285.53</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1314.1</v>
+        <v>1225.52</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>1310.92</v>
+        <v>5340.97</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>1821.61</v>
+        <v>1464.2</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>1056.15</v>
+        <v>1523</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>1638.4</v>
+        <v>3348</v>
       </c>
       <c r="P43" s="3" t="n">
-        <v>1660.35</v>
+        <v>2184.07</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>752.78</v>
+        <v>2346.5</v>
       </c>
       <c r="R43" s="3" t="n">
-        <v>15142.09</v>
+        <v>27669.43</v>
       </c>
     </row>
     <row r="44">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Insurance: staff medical insurance → OHF</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4505,52 +4505,52 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back-office staff on-costs</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>courier, flags/badges, miscellaneous</t>
+          <t>staff on-cost; monthly headcount key (Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr); ruling 13 Oct 2026, Option 3</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>2138.76</v>
+        <v>2188.2</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>1089.69</v>
+        <v>1991.55</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>1123.01</v>
+        <v>2389.86</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>3789.07</v>
+        <v>2389.86</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>1320.49</v>
+        <v>2452.83</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>989.6799999999999</v>
+        <v>2698.11</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>1127.98</v>
+        <v>1785.91</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>1253.75</v>
+        <v>717.3</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>508.94</v>
+        <v>807.72</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>264.83</v>
+        <v>822.6799999999999</v>
       </c>
       <c r="P44" s="3" t="n">
-        <v>316.45</v>
+        <v>849.35</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>88.53</v>
+        <v>867.98</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>14011.18</v>
+        <v>19961.35</v>
       </c>
     </row>
     <row r="45">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Insurance: on-cost → OHF</t>
+          <t>Fines</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4571,52 +4571,52 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Overhead — back-office staff on-costs</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>prepaid insurance amortised (staff medical insurance, Daman); staff on-cost split by the month's salary share of Indirect/RAP, Indirect /INS, Indirect /Management, Indirect /Purchase, Indirect/Accounts, Indirect it, Indirect/ Hr (ruling 13 Oct 2026)</t>
+          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>1055.81</v>
+        <v>1635</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>881.28</v>
+        <v>263</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>1050.52</v>
+        <v>0</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>1516.22</v>
+        <v>1278</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>1448.93</v>
+        <v>0</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>1579.89</v>
+        <v>1031</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>1382.3</v>
+        <v>0</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>546.45</v>
+        <v>8435.120000000001</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>565.1799999999999</v>
+        <v>1503</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>503.13</v>
+        <v>0</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>587.6900000000001</v>
+        <v>2242.91</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>540.89</v>
+        <v>625</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>11658.29</v>
+        <v>17013.03</v>
       </c>
     </row>
     <row r="46">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Pantry</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4637,52 +4637,52 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>stationery, printer ink, newspapers</t>
+          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>783.13</v>
+        <v>1576.08</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>449.05</v>
+        <v>1074.12</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>373</v>
+        <v>748.9299999999999</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>1618.98</v>
+        <v>1483.1</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>404.77</v>
+        <v>705.55</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1228.67</v>
+        <v>1314.1</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>340.61</v>
+        <v>1310.92</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>481.01</v>
+        <v>1821.61</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>1156.65</v>
+        <v>1056.15</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>440.57</v>
+        <v>1638.4</v>
       </c>
       <c r="P46" s="3" t="n">
-        <v>237.4</v>
+        <v>1660.35</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>375.55</v>
+        <v>752.78</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>7889.39</v>
+        <v>15142.09</v>
       </c>
     </row>
     <row r="47">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Claim Rejection</t>
+          <t>Other Expenses</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -4703,63 +4703,63 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>written-off rejected claims</t>
+          <t>courier, flags/badges, miscellaneous</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>0</v>
+        <v>2138.76</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>0</v>
+        <v>1089.69</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>844.2</v>
+        <v>1123.01</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>0</v>
+        <v>3789.07</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0</v>
+        <v>1320.49</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>245</v>
+        <v>989.6799999999999</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0</v>
+        <v>1127.98</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0</v>
+        <v>1253.75</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>1005</v>
+        <v>508.94</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>-32</v>
+        <v>264.83</v>
       </c>
       <c r="P47" s="3" t="n">
-        <v>1235</v>
+        <v>316.45</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>105</v>
+        <v>88.53</v>
       </c>
       <c r="R47" s="3" t="n">
-        <v>3402.2</v>
+        <v>14011.18</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): OHF</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4769,63 +4769,63 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>pantry and stationery issued from stock</t>
+          <t>stationery, printer ink, newspapers</t>
         </is>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1007.8</v>
+        <v>783.13</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0</v>
+        <v>449.05</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0</v>
+        <v>373</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0</v>
+        <v>1618.98</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0</v>
+        <v>404.77</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0</v>
+        <v>1228.67</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0</v>
+        <v>340.61</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0</v>
+        <v>481.01</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0</v>
+        <v>1156.65</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0</v>
+        <v>440.57</v>
       </c>
       <c r="P48" s="3" t="n">
-        <v>0</v>
+        <v>237.4</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>0</v>
+        <v>375.55</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>1007.8</v>
+        <v>7889.39</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect it</t>
+          <t>Claim Rejection</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4835,12 +4835,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Overhead — IT</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>written-off rejected claims</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
@@ -4850,7 +4850,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>0</v>
+        <v>844.2</v>
       </c>
       <c r="I49" s="3" t="n">
         <v>0</v>
@@ -4859,7 +4859,7 @@
         <v>0</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="L49" s="3" t="n">
         <v>0</v>
@@ -4868,30 +4868,30 @@
         <v>0</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>0</v>
+        <v>1005</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0</v>
+        <v>-32</v>
       </c>
       <c r="P49" s="3" t="n">
-        <v>0</v>
+        <v>1235</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>0</v>
+        <v>3402.2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Salary sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+          <t>Cost of Goods Sold (M01): OHF</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4901,16 +4901,16 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Overhead — HR</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>pantry and stationery issued from stock</t>
         </is>
       </c>
       <c r="F50" s="3" t="n">
-        <v>0</v>
+        <v>1007.8</v>
       </c>
       <c r="G50" s="3" t="n">
         <v>0</v>
@@ -4946,253 +4946,385 @@
         <v>0</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>0</v>
+        <v>1007.8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TB depreciation</t>
+          <t>Salary sheet</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Depreciation: furniture, office equipment, computers, software</t>
+          <t>Salaries &amp; Wages: Indirect it</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>OHDepreciation</t>
+          <t>OHF</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Overhead — facility / IT</t>
+          <t>Overhead — IT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="P51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>2524.8</v>
+        <v>0</v>
       </c>
       <c r="R51" s="3" t="n">
-        <v>30297.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Salary sheet</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Salaries &amp; Wages: Indirect/ Hr</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Overhead — HR</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TB depreciation</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Depreciation: furniture, office equipment, computers, software</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Overhead — facility / IT</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>fit-out, office equipment, computers, software (2025 charge 30,297.55)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="M53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="N53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="O53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="P53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="Q53" s="3" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="R53" s="3" t="n">
+        <v>30297.6</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Monthly sheet</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Third Party &amp; Professional Services</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>OHC</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Overhead — shared services</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>MySmyle Company EMR subscription, management consultancy and IT services (25,000/month) + Calibrate/Platform Technologies: services charged by a sister company = corporate/shared-services overhead</t>
         </is>
       </c>
-      <c r="F52" s="3" t="n">
+      <c r="F54" s="3" t="n">
         <v>8317</v>
       </c>
-      <c r="G52" s="3" t="n">
+      <c r="G54" s="3" t="n">
         <v>37300</v>
       </c>
-      <c r="H52" s="3" t="n">
+      <c r="H54" s="3" t="n">
         <v>62270</v>
       </c>
-      <c r="I52" s="3" t="n">
+      <c r="I54" s="3" t="n">
         <v>66480.95</v>
       </c>
-      <c r="J52" s="3" t="n">
+      <c r="J54" s="3" t="n">
         <v>2500</v>
       </c>
-      <c r="K52" s="3" t="n">
+      <c r="K54" s="3" t="n">
         <v>37375.73</v>
       </c>
-      <c r="L52" s="3" t="n">
+      <c r="L54" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="M52" s="3" t="n">
+      <c r="M54" s="3" t="n">
         <v>27500</v>
       </c>
-      <c r="N52" s="3" t="n">
+      <c r="N54" s="3" t="n">
         <v>28000</v>
       </c>
-      <c r="O52" s="3" t="n">
+      <c r="O54" s="3" t="n">
         <v>25500</v>
       </c>
-      <c r="P52" s="3" t="n">
+      <c r="P54" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="Q52" s="3" t="n">
+      <c r="Q54" s="3" t="n">
         <v>25104.5</v>
       </c>
-      <c r="R52" s="3" t="n">
+      <c r="R54" s="3" t="n">
         <v>370348.18</v>
       </c>
     </row>
-    <row r="53">
-      <c r="F53" s="3" t="n"/>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="n"/>
-      <c r="I53" s="3" t="n"/>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="3" t="n"/>
-      <c r="L53" s="3" t="n"/>
-      <c r="M53" s="3" t="n"/>
-      <c r="N53" s="3" t="n"/>
-      <c r="O53" s="3" t="n"/>
-      <c r="P53" s="3" t="n"/>
-      <c r="Q53" s="3" t="n"/>
-      <c r="R53" s="3" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-      <c r="B54" s="4" t="inlineStr">
+    <row r="55">
+      <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
+      <c r="I55" s="3" t="n"/>
+      <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
+      <c r="L55" s="3" t="n"/>
+      <c r="M55" s="3" t="n"/>
+      <c r="N55" s="3" t="n"/>
+      <c r="O55" s="3" t="n"/>
+      <c r="P55" s="3" t="n"/>
+      <c r="Q55" s="3" t="n"/>
+      <c r="R55" s="3" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr"/>
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>TOTAL mapped</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr"/>
-      <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="5" t="n">
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="5" t="n">
         <v>511302.3</v>
       </c>
-      <c r="G54" s="5" t="n">
+      <c r="G56" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H54" s="5" t="n">
+      <c r="H56" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I54" s="5" t="n">
+      <c r="I56" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J54" s="5" t="n">
+      <c r="J56" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K54" s="5" t="n">
+      <c r="K56" s="5" t="n">
         <v>616494.08</v>
       </c>
-      <c r="L54" s="5" t="n">
+      <c r="L56" s="5" t="n">
         <v>480166.81</v>
       </c>
-      <c r="M54" s="5" t="n">
+      <c r="M56" s="5" t="n">
         <v>526990.09</v>
       </c>
-      <c r="N54" s="5" t="n">
+      <c r="N56" s="5" t="n">
         <v>509542.04</v>
       </c>
-      <c r="O54" s="5" t="n">
+      <c r="O56" s="5" t="n">
         <v>546725.96</v>
       </c>
-      <c r="P54" s="5" t="n">
+      <c r="P56" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q54" s="5" t="n">
+      <c r="Q56" s="5" t="n">
         <v>623033.72</v>
       </c>
-      <c r="R54" s="5" t="n">
+      <c r="R56" s="5" t="n">
         <v>6453401.91</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr"/>
-      <c r="B55" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>Ledger (locked)</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="5" t="n">
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="5" t="n">
         <v>511302.3</v>
       </c>
-      <c r="G55" s="5" t="n">
+      <c r="G57" s="5" t="n">
         <v>532341.65</v>
       </c>
-      <c r="H55" s="5" t="n">
+      <c r="H57" s="5" t="n">
         <v>606868.87</v>
       </c>
-      <c r="I55" s="5" t="n">
+      <c r="I57" s="5" t="n">
         <v>518123.67</v>
       </c>
-      <c r="J55" s="5" t="n">
+      <c r="J57" s="5" t="n">
         <v>488066.69</v>
       </c>
-      <c r="K55" s="5" t="n">
+      <c r="K57" s="5" t="n">
         <v>616494.09</v>
       </c>
-      <c r="L55" s="5" t="n">
+      <c r="L57" s="5" t="n">
         <v>480166.82</v>
       </c>
-      <c r="M55" s="5" t="n">
+      <c r="M57" s="5" t="n">
         <v>526990.1</v>
       </c>
-      <c r="N55" s="5" t="n">
+      <c r="N57" s="5" t="n">
         <v>509542.05</v>
       </c>
-      <c r="O55" s="5" t="n">
+      <c r="O57" s="5" t="n">
         <v>546725.98</v>
       </c>
-      <c r="P55" s="5" t="n">
+      <c r="P57" s="5" t="n">
         <v>493746.03</v>
       </c>
-      <c r="Q55" s="5" t="n">
+      <c r="Q57" s="5" t="n">
         <v>623033.73</v>
       </c>
-      <c r="R55" s="5" t="n">
+      <c r="R57" s="5" t="n">
         <v>6453401.98</v>
       </c>
     </row>
@@ -5230,7 +5362,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q2. Staff on-costs (Staff Qualification And Education 889,431.99 in full; Insurance 50,409.29 in full; clinician licences 34,349.57 and visas / labour 145,165.32 out of Legal &amp; Professional) are split every month by the salary share of dentists / nurses / CSSD + technicians / back office, employees only (ruling 13 Oct 2026). The rest of Legal &amp; Professional (facility licences, accreditation, trade licence, civil defence, tenancy) stays OHF.</t>
+          <t>Q2. Staff on-costs, employees only (ruling 13 Oct 2026, Option 3 by nature of the cost): benefits / bonus / end-of-service / training (889,431.99) by the month's salary share of dentists / nurses / CSSD + technicians / back office; visas / labour (145,165.32) and staff medical insurance (50,409.29) by the month's headcount; clinician licences (34,349.57) to dentists and licensed nurses by headcount. The rest of Legal &amp; Professional (facility licences, accreditation, trade licence, civil defence, tenancy) stays OHF.</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5390,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Overhead ratio by month: 01 25.7%, 02 26.7%, 03 30.0%, 04 36.9%, 05 28.0%, 06 35.2%, 07 34.8%, 08 35.1%, 09 36.9%, 10 32.5%, 11 36.9%, 12 29.7%; FY2025 32.3% (DOH band 20% to under 50%)</t>
+          <t>Overhead ratio by month: 01 26.7%, 02 27.1%, 03 30.5%, 04 37.2%, 05 28.5%, 06 35.9%, 07 34.9%, 08 35.2%, 09 37.0%, 10 32.7%, 11 37.1%, 12 29.9%; FY2025 32.7% (DOH band 20% to under 50%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Full-year stock movement: split cost of goods sold for all twelve months on the three value bases; rulings on April, August and external lab; rebuild all twelve corrected files and reports
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/input/Ledger_by_Cost_Type_FY2025.xlsx
+++ b/input/Ledger_by_Cost_Type_FY2025.xlsx
@@ -868,37 +868,37 @@
         <v>1252</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>1097</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>1063.15</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>1063.15</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0</v>
+        <v>1014</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
+        <v>1506</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>1359</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>2243.5</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
+        <v>1145.54</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0</v>
+        <v>1203.75</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>782.9</v>
       </c>
       <c r="O8" s="3">
         <f>SUM(C8:N8)</f>
@@ -920,37 +920,37 @@
         <v>70074.94</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>18659.88</v>
+        <v>59229.44</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45146.24</v>
+        <v>88151.42</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>27454.24</v>
+        <v>70459.42</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>22166.68</v>
+        <v>63639.05</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>13158.04</v>
+        <v>53007.03</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23899.96</v>
+        <v>46524.6</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>31652.81</v>
+        <v>69988.98</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>19158.99</v>
+        <v>57602.32</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>20817.63</v>
+        <v>49525.36</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>36588.73</v>
+        <v>53926.7</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>39938.75</v>
+        <v>68940.98</v>
       </c>
       <c r="O9" s="3">
         <f>SUM(C9:N9)</f>
@@ -972,37 +972,37 @@
         <v>31662.75</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>70788.92999999999</v>
+        <v>28366.96</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>75671.17</v>
+        <v>30966.43</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>75671.17</v>
+        <v>30966.43</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>67508.86</v>
+        <v>24043.48</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65224.37</v>
+        <v>23064.38</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>50882.71</v>
+        <v>26049.57</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>71569.74000000001</v>
+        <v>30284.7</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>65977.17</v>
+        <v>25239.34</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>55565.68</v>
+        <v>25007.41</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>45169.67</v>
+        <v>25059.69</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>60394.62</v>
+        <v>23384.86</v>
       </c>
       <c r="O10" s="3">
         <f>SUM(C10:N10)</f>
@@ -1180,37 +1180,37 @@
         <v>125596.78</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>104364.95</v>
+        <v>105120.36</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>120047.2</v>
+        <v>120683.61</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>123705</v>
+        <v>124341.41</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>134056.35</v>
+        <v>134897.36</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>181154.59</v>
+        <v>182451.59</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>140052.85</v>
+        <v>140755.35</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>155505.23</v>
+        <v>157095.1</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>158108.08</v>
+        <v>158159.08</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>150575.63</v>
+        <v>151280.63</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>155870.88</v>
+        <v>157439.14</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>158965.77</v>
+        <v>166190.4</v>
       </c>
       <c r="O14" s="3">
         <f>SUM(C14:N14)</f>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Pharmacy</t>
+          <t>Cost of Goods Sold (M01, M02, M03, M04, M05, M06, M07, M08, M09, M10, M11, M12): Pharmacy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2801,51 +2801,51 @@
         <v>1252</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0</v>
+        <v>1097</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0</v>
+        <v>1063.15</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0</v>
+        <v>1063.15</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0</v>
+        <v>1014</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0</v>
+        <v>1506</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0</v>
+        <v>1359</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0</v>
+        <v>2243.5</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0</v>
+        <v>1145.54</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0</v>
+        <v>1203.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0</v>
+        <v>782.9</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>1252</v>
+        <v>14881.99</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Internal LAB</t>
+          <t>Cost of Goods Sold (M01, M02, M03, M04, M05, M06, M07, M08, M09, M10, M11, M12): Prostheses</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2855,63 +2855,63 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Direct — prostheses</t>
+          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
+          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>68204.94</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>18259.88</v>
+        <v>59029.44</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>21431.24</v>
+        <v>71721.42</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>21431.24</v>
+        <v>66171.42</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>7316.68</v>
+        <v>56214.05</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>13158.04</v>
+        <v>53007.03</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>13819.96</v>
+        <v>41254.6</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>20017.81</v>
+        <v>63607.98</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>16858.99</v>
+        <v>56452.32</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>18917.63</v>
+        <v>48575.36</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>15006.23</v>
+        <v>43331.7</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>15194.75</v>
+        <v>56754.73</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>181412.45</v>
+        <v>684324.99</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): Prostheses</t>
+          <t>External Lab</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2921,63 +2921,63 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Direct — prostheses (implants + in-house lab + external lab)</t>
+          <t>Direct — prostheses</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>implant fixtures (net of internal returns), healing/cover screws, abutments, implant impression tools, bone-graft materials; in-house CAD/CAM materials (blocks, blanks, 3D inks, stone, milling tools); external lab invoices</t>
+          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>68204.94</v>
+        <v>1870</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0</v>
+        <v>16430</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0</v>
+        <v>4288</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0</v>
+        <v>7425</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0</v>
+        <v>5270</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0</v>
+        <v>6381</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0</v>
+        <v>1150</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0</v>
+        <v>10595</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0</v>
+        <v>12186.25</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>68204.94</v>
+        <v>66745.25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>External Lab</t>
+          <t>Cost of Goods Sold: Internal LAB</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2992,47 +2992,47 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>outsourced dental laboratory invoices (expense head) — prostheses bought from external labs (ruling 13 Oct 2026)</t>
+          <t>in-house CAD/CAM prosthesis materials (ruling 13 Oct 2026: no laboratory; prostheses)</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1870</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>16430</v>
+        <v>0</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>4288</v>
+        <v>0</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>7425</v>
+        <v>0</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>5270</v>
+        <v>0</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>6381</v>
+        <v>0</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>10595</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>12186.25</v>
+        <v>0</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>66745.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3065,51 +3065,51 @@
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>7285</v>
+        <v>0</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>1735</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>7425</v>
+        <v>0</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>4810</v>
+        <v>0</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>5254</v>
+        <v>0</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>10987.5</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>12557.75</v>
+        <v>0</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>52354.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Consumption sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -( Dr</t>
+          <t>Cost of Goods Sold (M01, M02, M03, M04, M05, M06, M07, M08, M09, M10, M11, M12): MS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3119,52 +3119,52 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries</t>
+          <t>Direct — dental surgeries / CSSD</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>clinical consumables issued to the dental surgeries</t>
+          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0</v>
+        <v>31662.75</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>67171.58</v>
+        <v>28366.96</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>70803.81</v>
+        <v>30966.43</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>70803.81</v>
+        <v>30966.43</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>63371.43</v>
+        <v>24043.48</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>61129.96</v>
+        <v>23064.38</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>46785.8</v>
+        <v>26049.57</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>67034.7</v>
+        <v>30284.7</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>62943.56</v>
+        <v>25239.34</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>51591.7</v>
+        <v>25007.41</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>39376.22</v>
+        <v>25059.69</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>50594.58</v>
+        <v>23384.86</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>651607.15</v>
+        <v>324096</v>
       </c>
     </row>
     <row r="24">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
+          <t>Cost of Goods Sold: Consumables -( Dr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3185,63 +3185,63 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Direct — CSSD</t>
+          <t>Direct — dental surgeries</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>sterilisation and vital-signs consumables</t>
+          <t>clinical consumables issued to the dental surgeries</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>3617.35</v>
+        <v>0</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>4867.36</v>
+        <v>0</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>4137.43</v>
+        <v>0</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>4094.41</v>
+        <v>0</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>4096.91</v>
+        <v>0</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>4535.04</v>
+        <v>0</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>3033.61</v>
+        <v>0</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>3973.98</v>
+        <v>0</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>5793.45</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>9800.040000000001</v>
+        <v>0</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>52816.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Consumption sheet</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): MS</t>
+          <t>Cost of Goods Sold: Consumables -  ( CSSD</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3251,16 +3251,16 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Direct — dental surgeries / CSSD</t>
+          <t>Direct — CSSD</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>restorative, endodontic, burs, impression, bleaching, surgical, infection-control supplies, needles/syringes, hand instruments</t>
+          <t>sterilisation and vital-signs consumables</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>31662.75</v>
+        <v>0</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>0</v>
@@ -3296,7 +3296,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>31662.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4556,12 +4556,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Monthly sheet</t>
+          <t>Stock movement</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Fines</t>
+          <t>Cost of Goods Sold (M01, M02, M03, M04, M05, M06, M07, M08, M09, M10, M11, M12): OHF</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4571,52 +4571,52 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
+          <t>pantry and stationery issued from stock</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>1635</v>
+        <v>1007.8</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>263</v>
+        <v>755.4</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0</v>
+        <v>636.4</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>1278</v>
+        <v>636.4</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0</v>
+        <v>841</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>1031</v>
+        <v>1297</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0</v>
+        <v>702.5</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>8435.120000000001</v>
+        <v>1589.87</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>1503</v>
+        <v>51</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0</v>
+        <v>705</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>2242.91</v>
+        <v>1568.26</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>625</v>
+        <v>7224.63</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>17013.03</v>
+        <v>17015.26</v>
       </c>
     </row>
     <row r="46">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Pantry</t>
+          <t>Fines</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4637,52 +4637,52 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
+          <t>regulatory and traffic fines (kept: Standard 3.1.1 takes all GL expenses except balance-sheet items)</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>1576.08</v>
+        <v>1635</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>1074.12</v>
+        <v>263</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>748.9299999999999</v>
+        <v>0</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>1483.1</v>
+        <v>1278</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>705.55</v>
+        <v>0</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1314.1</v>
+        <v>1031</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>1310.92</v>
+        <v>0</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>1821.61</v>
+        <v>8435.120000000001</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>1056.15</v>
+        <v>1503</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>1638.4</v>
+        <v>0</v>
       </c>
       <c r="P46" s="3" t="n">
-        <v>1660.35</v>
+        <v>2242.91</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>752.78</v>
+        <v>625</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>15142.09</v>
+        <v>17013.03</v>
       </c>
     </row>
     <row r="47">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Other Expenses</t>
+          <t>Pantry</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -4703,52 +4703,52 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Overhead — administration</t>
+          <t>Overhead — back office</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>courier, flags/badges, miscellaneous</t>
+          <t>pantry, water, cleaning products (staff and patient refreshments)</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>2138.76</v>
+        <v>1576.08</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>1089.69</v>
+        <v>1074.12</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>1123.01</v>
+        <v>748.9299999999999</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>3789.07</v>
+        <v>1483.1</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>1320.49</v>
+        <v>705.55</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>989.6799999999999</v>
+        <v>1314.1</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>1127.98</v>
+        <v>1310.92</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>1253.75</v>
+        <v>1821.61</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>508.94</v>
+        <v>1056.15</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>264.83</v>
+        <v>1638.4</v>
       </c>
       <c r="P47" s="3" t="n">
-        <v>316.45</v>
+        <v>1660.35</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>88.53</v>
+        <v>752.78</v>
       </c>
       <c r="R47" s="3" t="n">
-        <v>14011.18</v>
+        <v>15142.09</v>
       </c>
     </row>
     <row r="48">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Other Expenses</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4774,47 +4774,47 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>stationery, printer ink, newspapers</t>
+          <t>courier, flags/badges, miscellaneous</t>
         </is>
       </c>
       <c r="F48" s="3" t="n">
-        <v>783.13</v>
+        <v>2138.76</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>449.05</v>
+        <v>1089.69</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>373</v>
+        <v>1123.01</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>1618.98</v>
+        <v>3789.07</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>404.77</v>
+        <v>1320.49</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1228.67</v>
+        <v>989.6799999999999</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>340.61</v>
+        <v>1127.98</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>481.01</v>
+        <v>1253.75</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>1156.65</v>
+        <v>508.94</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>440.57</v>
+        <v>264.83</v>
       </c>
       <c r="P48" s="3" t="n">
-        <v>237.4</v>
+        <v>316.45</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>375.55</v>
+        <v>88.53</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>7889.39</v>
+        <v>14011.18</v>
       </c>
     </row>
     <row r="49">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Claim Rejection</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4835,63 +4835,63 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Overhead — patient administration</t>
+          <t>Overhead — administration</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>written-off rejected claims</t>
+          <t>stationery, printer ink, newspapers</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>0</v>
+        <v>783.13</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0</v>
+        <v>449.05</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>844.2</v>
+        <v>373</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>0</v>
+        <v>1618.98</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>0</v>
+        <v>404.77</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>245</v>
+        <v>1228.67</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0</v>
+        <v>340.61</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0</v>
+        <v>481.01</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>1005</v>
+        <v>1156.65</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>-32</v>
+        <v>440.57</v>
       </c>
       <c r="P49" s="3" t="n">
-        <v>1235</v>
+        <v>237.4</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>105</v>
+        <v>375.55</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>3402.2</v>
+        <v>7889.39</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Stock movement</t>
+          <t>Monthly sheet</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold (M01): OHF</t>
+          <t>Claim Rejection</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4901,22 +4901,22 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Overhead — back office</t>
+          <t>Overhead — patient administration</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>pantry and stationery issued from stock</t>
+          <t>written-off rejected claims</t>
         </is>
       </c>
       <c r="F50" s="3" t="n">
-        <v>1007.8</v>
+        <v>0</v>
       </c>
       <c r="G50" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>0</v>
+        <v>844.2</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>0</v>
@@ -4925,7 +4925,7 @@
         <v>0</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="L50" s="3" t="n">
         <v>0</v>
@@ -4934,19 +4934,19 @@
         <v>0</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>0</v>
+        <v>1005</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0</v>
+        <v>-32</v>
       </c>
       <c r="P50" s="3" t="n">
-        <v>0</v>
+        <v>1235</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>1007.8</v>
+        <v>3402.2</v>
       </c>
     </row>
     <row r="51">
@@ -5242,16 +5242,16 @@
         <v>511302.3</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>532341.65</v>
+        <v>532341.64</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>606868.87</v>
+        <v>606868.86</v>
       </c>
       <c r="I56" s="5" t="n">
-        <v>518123.67</v>
+        <v>518123.66</v>
       </c>
       <c r="J56" s="5" t="n">
-        <v>488066.69</v>
+        <v>488066.68</v>
       </c>
       <c r="K56" s="5" t="n">
         <v>616494.08</v>
@@ -5275,7 +5275,7 @@
         <v>623033.72</v>
       </c>
       <c r="R56" s="5" t="n">
-        <v>6453401.91</v>
+        <v>6453401.87</v>
       </c>
     </row>
     <row r="57">
@@ -5339,7 +5339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -5390,7 +5390,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Overhead ratio by month: 01 26.7%, 02 27.1%, 03 30.5%, 04 37.2%, 05 28.5%, 06 35.9%, 07 34.9%, 08 35.2%, 09 37.0%, 10 32.7%, 11 37.1%, 12 29.9%; FY2025 32.7% (DOH band 20% to under 50%)</t>
+          <t>Overhead ratio by month: 01 26.7%, 02 27.2%, 03 30.6%, 04 37.3%, 05 28.7%, 06 36.1%, 07 35.0%, 08 35.5%, 09 37.0%, 10 32.8%, 11 37.5%, 12 31.1%; FY2025 32.9% (DOH band 20% to under 50%)</t>
         </is>
       </c>
     </row>
@@ -5404,110 +5404,166 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 2: split 89248.81 != Monthly 89248.80</t>
+          <t>month 1: stock movement 102,127.48 vs Cost of Goods Sold 102,127.49: +0.01 placed on MS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 3: split 104387.41 != Monthly 104387.40</t>
+          <t>month 6: stock movement 78,382.40 vs Cost of Goods Sold 78,382.41: +0.01 placed on MS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 4: split 98837.41 != Monthly 98837.40</t>
+          <t>month 7: stock movement 69,512.68 vs Cost of Goods Sold 69,512.67: -0.01 placed on MS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold month 5: split 82250.54 != Monthly 82250.53</t>
+          <t>month 8: stock movement 96,409.73 vs Cost of Goods Sold 96,841.55: +431.82 placed on MS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>month 6: mapped total 616494.08 != ledger 616494.09 (-0.01)</t>
+          <t>month 2: mapped total 532341.64 != ledger 532341.65 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>month 7: mapped total 480166.81 != ledger 480166.82 (-0.01)</t>
+          <t>month 3: mapped total 606868.86 != ledger 606868.87 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>month 8: mapped total 526990.09 != ledger 526990.10 (-0.01)</t>
+          <t>month 4: mapped total 518123.66 != ledger 518123.67 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>month 9: mapped total 509542.04 != ledger 509542.05 (-0.01)</t>
+          <t>month 5: mapped total 488066.68 != ledger 488066.69 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>month 10: mapped total 546725.96 != ledger 546725.98 (-0.02)</t>
+          <t>month 6: mapped total 616494.08 != ledger 616494.09 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>month 12: mapped total 623033.72 != ledger 623033.73 (-0.01)</t>
+          <t>month 7: mapped total 480166.81 != ledger 480166.82 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>month 6: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 8: mapped total 526990.09 != ledger 526990.10 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>month 7: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 9: mapped total 509542.04 != ledger 509542.05 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>month 8: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 10: mapped total 546725.96 != ledger 546725.98 (-0.02)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>month 9: +0.01 added to OHF to tie to the locked ledger</t>
+          <t>month 12: mapped total 623033.72 != ledger 623033.73 (-0.01)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>month 10: +0.02 added to OHF to tie to the locked ledger</t>
+          <t>month 2: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
+        <is>
+          <t>month 3: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>month 4: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>month 5: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>month 6: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>month 7: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>month 8: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>month 9: +0.01 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>month 10: +0.02 added to OHF to tie to the locked ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>month 12: +0.01 added to OHF to tie to the locked ledger</t>
         </is>
@@ -5524,7 +5580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -5540,238 +5596,2954 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   05- Medical Electronic Devices (Restorative, Perio, Endo, Implants, Ortho…)    5,500.00</t>
+          <t>M01: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   05- Medical Electronic Devices (Restorative, P      5,500.00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo, Implants,Ortho…)       83.33</t>
+          <t>M01: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo         83.33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   345.28</t>
+          <t>M01: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   345.28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,993.20</t>
+          <t>M01: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,993.20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,477.50</t>
+          <t>M01: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,477.50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,007.00</t>
+          <t>M01: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,007.00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        540.65</t>
+          <t>M01: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        540.65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   338.00</t>
+          <t>M01: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   338.00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          806.00</t>
+          <t>M01: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          806.00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,552.50</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,552.50</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            756.62</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            756.62</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      4,441.00</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      4,441.00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,630.33</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,630.33</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     710.82</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     710.82</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   690.50</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   690.50</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,700.00</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,700.00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            90.00</t>
+          <t>M01: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            90.00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   847.80</t>
+          <t>M01: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   847.80</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  160.00</t>
+          <t>M01: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  160.00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                682.00</t>
+          <t>M01: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                682.00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         570.00</t>
+          <t>M01: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         570.00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               27,500.00</t>
+          <t>M01: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               27,500.00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           3,699.00</t>
+          <t>M01: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           3,699.00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       6,652.00</t>
+          <t>M01: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       6,652.00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               960.00</t>
+          <t>M01: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               960.00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             13,985.00</t>
+          <t>M01: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             13,985.00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           130.00</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           130.00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,889.75</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,889.75</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   1,875.00</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   1,875.00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              5,000.00</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              5,000.00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   58.19</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   58.19</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        985.00</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        985.00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessories     1,601.00</t>
+          <t>M01: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      1,601.00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Movement Jan 2025: Prostheses  External LAB invoices (P&amp;L line, not stock)                                        1,870.00</t>
+          <t>M01: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            1,870.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>M02: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories       2,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>M02: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo        294.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>M02: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                    52.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>M02: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,713.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>M02: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   1,838.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>M02: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,740.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>M02: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        556.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>M02: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   348.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>M02: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          494.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               530.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies          1,104.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      6,051.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           7,108.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     424.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                 1,726.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                1,974.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>M02: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           410.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>M02: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   652.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>M02: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  103.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>M02: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                407.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>M02: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         690.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               28,750.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           1,096.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       1,750.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies             2,525.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              9,150.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   4,870.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   3,025.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              1,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  154.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                      3,700.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      2,024.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>M02: Prostheses 06- Laboratory- (LAB)                           09- External Lab &amp; Invisaligns                        285.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>M02: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                              200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>M03: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo      4,650.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>M03: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                    17.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>M03: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,549.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>M03: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,033.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>M03: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,806.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>M03: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        643.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>M03: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   310.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>M03: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          816.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               905.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            450.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      5,920.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,666.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     611.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   984.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                3,226.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>M03: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           176.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>M03: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   556.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>M03: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                   80.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>M03: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                502.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>M03: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              02- Medicines &amp; Medicaments                            51.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>M03: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         510.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               21,250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           1,233.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       8,355.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies             1,435.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              7,850.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           370.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   2,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              6,220.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  141.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        940.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie        996.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>M03: Prostheses 06- Laboratory- (LAB)                           09- External Lab &amp; Invisaligns                     10,145.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>M03: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            7,285.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>M04: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo      4,650.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>M04: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                    17.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>M04: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,549.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>M04: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,033.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>M04: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,806.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>M04: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        643.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>M04: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   310.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>M04: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          816.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               905.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            450.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      5,920.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,666.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     611.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   984.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                3,226.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>M04: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           176.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>M04: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   556.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>M04: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                   80.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>M04: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                502.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>M04: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              02- Medicines &amp; Medicaments                            51.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>M04: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         510.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               21,250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                           1,233.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       8,355.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies             1,435.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              7,850.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           370.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   3,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   2,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              6,220.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  141.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        940.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie        996.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>M04: Prostheses 06- Laboratory- (LAB)                           09- External Lab &amp; Invisaligns                     10,145.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>M04: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            1,735.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>M05: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories         390.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>M05: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo        173.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>M05: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                    52.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>M05: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              2,174.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>M05: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,233.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>M05: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,792.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>M05: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        516.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>M05: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   366.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>M05: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          441.45</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               570.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            698.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      5,727.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,893.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     197.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   970.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                     400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                2,019.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>M05: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           426.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>M05: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   108.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>M05: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  733.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>M05: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                462.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>M05: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         690.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               32,196.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 05- Implants- (IMPL)                            03- Abutments                                         700.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               640.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              8,935.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   3,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              2,560.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   52.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        185.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>M05: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie        520.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>M05: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            7,425.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>M06: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories         100.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>M06: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   218.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>M06: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,628.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>M06: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   1,879.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>M06: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,546.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>M06: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        839.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>M06: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   274.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>M06: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          512.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               470.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            944.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      7,007.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           3,743.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                   1,267.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   597.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   2,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>M06: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            37.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>M06: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                 1,062.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>M06: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  235.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>M06: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                594.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>M06: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         420.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               30,303.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       1,750.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              8,512.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   2,890.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   3,465.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              3,585.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  176.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        640.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      1,460.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>M06: Prostheses 06- Laboratory- (LAB)                           08- Sand Blasting Materials &amp; Supplies                225.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>M07: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories       1,356.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>M07: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                    55.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>M07: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              2,797.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>M07: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,488.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>M07: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,315.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>M07: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        642.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>M07: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   394.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>M07: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          547.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               700.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies          1,092.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      5,406.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,991.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     665.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   300.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                  557.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>M07: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           140.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>M07: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   350.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>M07: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  352.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>M07: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                576.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>M07: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         930.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               14,810.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                               0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       4,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies             1,850.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              5,800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           265.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   4,212.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                     905.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              2,265.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   47.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        216.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>M07: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      1,572.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>M07: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            4,810.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>M08: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo        191.57</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>M08: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   131.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>M08: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              2,504.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>M08: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,269.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>M08: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,539.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>M08: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        949.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>M08: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   344.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>M08: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          386.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                             1,285.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            643.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies     11,469.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,211.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     506.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                 2,087.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                     400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                  710.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>M08: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           223.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>M08: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                 1,157.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>M08: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  432.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>M08: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                939.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>M08: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         420.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               24,674.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                             274.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       4,900.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              4,150.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories         4,761.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   5,272.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   3,015.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              3,090.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  166.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        766.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      2,034.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>M08: Prostheses 06- Laboratory- (LAB)                           09- External Lab &amp; Invisaligns                      5,250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>M08: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            5,254.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>M09: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   01- Dental Chairs &amp; Accessories                        50.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>M09: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories       1,477.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>M09: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo        250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>M09: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   08- Cssd, Triage, PCI Devices                           0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>M09: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   155.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>M09: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,600.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>M09: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,420.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>M09: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,972.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>M09: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        402.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>M09: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   300.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>M09: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          769.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               365.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            922.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      6,868.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           3,816.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     955.83</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                   449.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                     800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                1,551.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>M09: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           111.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>M09: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                    28.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>M09: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                   23.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>M09: Pharmacy   01- Medical &amp; LAB Devices. Instruments- (DEV)   07- Nitrous &amp; Oxygen Sedation                         135.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>M09: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                820.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>M09: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              02- Medicines &amp; Medicaments                            58.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>M09: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                       1,230.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               29,015.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                             411.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       2,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies                 0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              9,400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           01- Lab Devices, Instruments, &amp; Accessories           550.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   2,888.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   3,095.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              1,650.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   72.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                      3,568.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>M09: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie      2,152.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>M09: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                            1,150.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>M10: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   04- Hand Pieces, Scaler Devices &amp; Accessories         100.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>M10: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo         31.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>M10: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                  -279.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>M10: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              2,398.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>M10: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,721.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>M10: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      1,464.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>M10: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        546.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>M10: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   286.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>M10: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          954.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               900.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies          1,006.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      5,248.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           4,290.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     855.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                 1,220.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                     400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                2,096.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>M10: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways           188.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>M10: MS         05- Implants- (IMPL)                            06- Screwdrivers &amp; Drilling Kits                      580.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>M10: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                   610.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>M10: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                   95.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>M10: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                328.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>M10: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              02- Medicines &amp; Medicaments                           357.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>M10: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         458.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               18,497.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       3,450.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               305.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic             10,880.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   6,041.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   4,382.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              2,533.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                  240.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        777.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie        509.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>M10: Prostheses 06- Laboratory- (LAB)                           08- Sand Blasting Materials &amp; Supplies                  8.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>M10: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                              950.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>M11: MS         01- Medical &amp; LAB Devices. Instruments- (DEV)   06- Hand Instruments (Restorative, Perio, Endo        125.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>M11: MS         02- Drugs, Needles &amp; Triage- (DRG)              03- Vital Signs/ Emergency Supplies                   126.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>M11: MS         02- Drugs, Needles &amp; Triage- (DRG)              04- Needles &amp; Syringes                              1,387.56</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    01- Personal Protective Equipment                   2,086.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    02- Disinfectants &amp; Lubricants                      2,350.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    03- General &amp; Waste Management                        917.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    04- Wrapping &amp; Protective Materials                   406.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    05- Sterilization Monitoring                          547.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>M11: MS         03- Prevention &amp; Control of Infection- (PCI)    None                                                  112.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          01- Burs &amp; Stones Tools                               356.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          03- Scaling / Gingiva Materials &amp; Supplies            963.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          04- Restorative Fillings, Adhesives &amp; Supplies      6,380.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          05- Endodontic Materials &amp; Posts Supplies           5,812.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          06- Surgical Materials &amp; Supplies                     559.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          07- Impression Materials &amp; Supplies                 1,166.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          08- Bleaching Material &amp; Supplies                   1,200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          09- Orthodontic Materials &amp; Supplies                  537.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>M11: MS         04- Dental Materials &amp; Supplies- (DMS)          10- Patient Education Printouts &amp; Giveaways            25.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>M11: MS         05- Implants- (IMPL)                            06- Screwdrivers &amp; Drilling Kits                        0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>M11: OHF        07- Management of Information (MOI)             02- Laptop, Computer, Headphones &amp; Accessories        120.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>M11: OHF        08- Facility Management &amp; (FMS)                 07- Pantry Supplies                                 1,006.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>M11: OHF        08- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  441.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>M11: Pharmacy   01- Medical &amp; LAB Devices. Instruments- (DEV)   07- Nitrous &amp; Oxygen Sedation                          30.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>M11: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              01- Local Anaesthetics                                521.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>M11: Pharmacy   02- Drugs, Needles &amp; Triage- (DRG)              02- Medicines &amp; Medicaments                           202.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>M11: Pharmacy   04- Dental Materials &amp; Supplies- (DMS)          02- Nitrous &amp; Oxygen Sedation                         450.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                                9,022.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       1,575.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies             1,170.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              6,225.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           02- Dental Blocks                                   2,520.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           03- Dental Blanks                                   9,253.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           04- 3D Inks &amp; Supplies                              1,440.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           05- Vacuum Machine Plates &amp; Supplies                   70.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           06- Dental Stone, Stains &amp; Wax                        172.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>M11: Prostheses 06- Laboratory- (LAB)                           07- Lab Drilling / Milling  Tools &amp; Accessorie        895.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>M11: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                           10,987.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>M12: MS         01- Medical Devices and Instruments- (DEV)      03- Hand pieces, scaler devices &amp; accessories         158.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>M12: MS         01- Medical Devices and Instruments- (DEV)      04- Electronic Devices (Restorative, Perio, En        400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>M12: MS         02- Drugs, Needles and Triage- (DRG)            01- Local Anesthetics                                 733.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>M12: MS         02- Drugs, Needles and Triage- (DRG)            03- Vital Signs/ emergency Kits                       156.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>M12: MS         02- Drugs, Needles and Triage- (DRG)            04- Needles &amp; Syringes                              3,025.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>M12: MS         03- Prevention and Control of Infection- (PCI)  01- Personal Protective Equipment                   1,284.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>M12: MS         03- Prevention and Control of Infection- (PCI)  02- General &amp; Waste Management                      1,909.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>M12: MS         03- Prevention and Control of Infection- (PCI)  03- Wrapping &amp; Protective Materials                   810.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>M12: MS         03- Prevention and Control of Infection- (PCI)  04- Sterilizer Monitoring                             367.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        01- Burs &amp; Stones Tools                               425.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        03- Scaling / Gingiva Materials &amp; Supplies          1,229.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        04- Restorative Fillings, Adhesives &amp; Posts Ma      5,661.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        05- Endodontic Materials &amp; Supplies                 3,567.83</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        06- Surgical Materials &amp; Supplies                     419.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        07- Impression Materials &amp; Supplies                 1,593.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        08- Bleaching Material &amp; Supplies                       0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>M12: MS         04- Dental Materials and Supplies- (DMS)        09- Orthodontic Materials &amp; Supplies                1,395.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>M12: MS         05- Implants- (IMPL)                            06- Screwdriver                                       250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 02- Computer, Networking, &amp; Electronic Devices      2,664.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 03- Patient Education, Giveaways                       82.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 04- Pantry Device &amp; Supplies                        1,493.45</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 05- Equipment Safety and Maintenance tools            456.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 06- Photography &amp; Videography                       2,196.96</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>M12: OHF        07- Facility Management &amp; (FMS)                 08- Stationaries &amp; Printing Supplies                  331.47</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>M12: Pharmacy   01- Medical Devices and Instruments- (DEV)      06- Nitrous &amp; Oxygen Sedation                          15.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>M12: Pharmacy   02- Drugs, Needles and Triage- (DRG)            02- Medicaments                                       107.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>M12: Pharmacy   04- Dental Materials and Supplies- (DMS)        02- Nitrous &amp; Oxygen Sedation                         660.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 05- Implants- (IMPL)                            01- Implant Fixtures                               16,598.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 05- Implants- (IMPL)                            02- Healing &amp; Cover Screw                               0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 05- Implants- (IMPL)                            03- Abutments                                       1,690.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 05- Implants- (IMPL)                            04- Implant Impression Tools &amp; Supplies               160.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 05- Implants- (IMPL)                            05- Bone Grafting Materials, Synthetic              9,450.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           01- Dental Blocks                                   1,604.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           02- Dental Blanks                                   4,583.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           03- 3D Inks &amp; Supplies                              1,679.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           04- Vaccum Machine Plates &amp; Supplies                  127.66</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           05- Dental Stains,Stone &amp; Wax                         990.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           06- Lab Tools &amp; Accessories                         1,838.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>M12: Prostheses 06- Laboratory- (LAB)                           08- External Lab                                    5,475.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>M12: Prostheses  External LAB invoices (Consumption sheet, cash in hand, not stock)                           12,557.75</t>
         </is>
       </c>
     </row>

</xml_diff>